<commit_message>
backend talepler görsel okuma yapılıyor.
</commit_message>
<xml_diff>
--- a/backend/app/temp/mukayese_raporu.xlsx
+++ b/backend/app/temp/mukayese_raporu.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="97">
   <si>
     <t>TEKLİF KARŞILAŞTIRMA RAPORU</t>
   </si>
@@ -46,7 +46,7 @@
     <t>En Avantajlı Firma Dağılımı</t>
   </si>
   <si>
-    <t>A Firması: 6  C Firması: 2  B Firması: 2</t>
+    <t>C Firması: 8  B Firması: 2</t>
   </si>
   <si>
     <t>Para Birimi</t>
@@ -61,10 +61,10 @@
     <t>Rapor Tarihi</t>
   </si>
   <si>
-    <t>24.04.2026</t>
-  </si>
-  <si>
-    <t>17:18</t>
+    <t>25.04.2026</t>
+  </si>
+  <si>
+    <t>21:16</t>
   </si>
   <si>
     <t>Kur Bilgisi</t>
@@ -163,31 +163,34 @@
     <t>60</t>
   </si>
   <si>
-    <t>A Firması</t>
+    <t>C Firması</t>
+  </si>
+  <si>
+    <t>En düşük net fiyat</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>pdr003</t>
+  </si>
+  <si>
+    <t>silgi</t>
+  </si>
+  <si>
+    <t>60 gün</t>
+  </si>
+  <si>
+    <t>45</t>
   </si>
   <si>
     <t>En avantajlı vade</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>pdr003</t>
-  </si>
-  <si>
-    <t>silgi</t>
-  </si>
-  <si>
-    <t>60 gün</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
     <t>pdr004</t>
   </si>
   <si>
-    <t>yesil kalem</t>
+    <t>yeşil kalem</t>
   </si>
   <si>
     <t>hafta</t>
@@ -196,13 +199,13 @@
     <t>1 hafta</t>
   </si>
   <si>
-    <t>En düşük net fiyat</t>
+    <t>B Firması</t>
   </si>
   <si>
     <t>pdr006</t>
   </si>
   <si>
-    <t>yesil silgi</t>
+    <t>yeşil silgi</t>
   </si>
   <si>
     <t>2 hafta</t>
@@ -229,25 +232,19 @@
     <t>90</t>
   </si>
   <si>
-    <t>PDF-0002</t>
+    <t>pdr002</t>
   </si>
   <si>
     <t>defter</t>
   </si>
   <si>
-    <t>C Firması</t>
-  </si>
-  <si>
-    <t>PDF-0005</t>
+    <t>pdr005</t>
   </si>
   <si>
     <t>turuncu kalem</t>
   </si>
   <si>
-    <t>B Firması</t>
-  </si>
-  <si>
-    <t>PDF-0008</t>
+    <t>pdr008</t>
   </si>
   <si>
     <t>sözlük</t>
@@ -256,7 +253,7 @@
     <t>3-4 hafta</t>
   </si>
   <si>
-    <t>PDF-0010</t>
+    <t>pdr010</t>
   </si>
   <si>
     <t>kalem tıraş</t>
@@ -298,15 +295,15 @@
     <t>EŞLEŞTİRME UYARILARI</t>
   </si>
   <si>
-    <t>• pdr004 / yesil kalem → yesil kalem ~ yeşil kalem
-• pdr006 / yesil silgi → yesil silgi ~ yeşil silgi</t>
+    <t>• pdr004 / yeşil kalem → yesil kalem ~ yeşil kalem
+• pdr006 / yeşil silgi → yesil silgi ~ yeşil silgi</t>
   </si>
   <si>
     <t>NOTLAR</t>
   </si>
   <si>
     <t>• Net birim fiyat = Birim fiyat x (1 - iskonto%).
-• Net toplam = Net birim fiyat x firma adedi.
+• Net toplam = Net birim fiyat x talep edilen adet.
 • Para birimi dönüşümleri kur bilgisine göre yapılmıştır.
 • Bu rapor bilgilendirme amaçlıdır.</t>
   </si>
@@ -314,7 +311,7 @@
     <t>Rapor Oluşturan: Sistem</t>
   </si>
   <si>
-    <t>Rapor No: RPR-20260424-1718</t>
+    <t>Rapor No: RPR-20260425-2116</t>
   </si>
 </sst>
 </file>
@@ -539,16 +536,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1138,7 +1135,7 @@
         <v>44</v>
       </c>
       <c r="E10" s="13">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F10" s="15">
         <v>0.25</v>
@@ -1150,24 +1147,24 @@
         <v>10.272</v>
       </c>
       <c r="I10" s="15">
-        <v>10.272</v>
-      </c>
-      <c r="J10" s="16" t="s">
+        <v>102.72</v>
+      </c>
+      <c r="J10" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K10" s="16" t="s">
+      <c r="K10" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="L10" s="17">
+      <c r="L10" s="15">
         <v>0.3</v>
       </c>
-      <c r="M10" s="18">
+      <c r="M10" s="16">
         <v>0</v>
       </c>
-      <c r="N10" s="17">
+      <c r="N10" s="15">
         <v>11.76</v>
       </c>
-      <c r="O10" s="17">
+      <c r="O10" s="15">
         <v>117.6</v>
       </c>
       <c r="P10" s="13" t="s">
@@ -1188,20 +1185,20 @@
       <c r="U10" s="17">
         <v>95</v>
       </c>
-      <c r="V10" s="13" t="s">
+      <c r="V10" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="W10" s="13" t="s">
+      <c r="W10" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="X10" s="16" t="s">
+      <c r="X10" s="18" t="s">
         <v>49</v>
       </c>
       <c r="Y10" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="Z10" s="15">
-        <v>10.272</v>
+      <c r="Z10" s="17">
+        <v>95</v>
       </c>
       <c r="AA10" s="14" t="s">
         <v>51</v>
@@ -1221,7 +1218,7 @@
         <v>44</v>
       </c>
       <c r="E11" s="13">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="F11" s="15">
         <v>1.4</v>
@@ -1233,24 +1230,24 @@
         <v>59.92</v>
       </c>
       <c r="I11" s="15">
-        <v>179.76</v>
-      </c>
-      <c r="J11" s="16" t="s">
+        <v>1797.6</v>
+      </c>
+      <c r="J11" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="K11" s="16" t="s">
+      <c r="K11" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="17">
+      <c r="L11" s="15">
         <v>1.1</v>
       </c>
-      <c r="M11" s="18">
+      <c r="M11" s="16">
         <v>0</v>
       </c>
-      <c r="N11" s="17">
+      <c r="N11" s="15">
         <v>43.12</v>
       </c>
-      <c r="O11" s="17">
+      <c r="O11" s="15">
         <v>1293.6</v>
       </c>
       <c r="P11" s="13" t="s">
@@ -1271,20 +1268,20 @@
       <c r="U11" s="17">
         <v>1323</v>
       </c>
-      <c r="V11" s="13" t="s">
+      <c r="V11" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="W11" s="13" t="s">
+      <c r="W11" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="X11" s="16" t="s">
+      <c r="X11" s="18" t="s">
         <v>49</v>
       </c>
       <c r="Y11" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z11" s="15">
-        <v>179.76</v>
+        <v>56</v>
+      </c>
+      <c r="Z11" s="17">
+        <v>1323</v>
       </c>
       <c r="AA11" s="14" t="s">
         <v>51</v>
@@ -1295,16 +1292,16 @@
         <v>3</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E12" s="13">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F12" s="15">
         <v>1.75</v>
@@ -1316,13 +1313,13 @@
         <v>71.155</v>
       </c>
       <c r="I12" s="15">
-        <v>284.62</v>
-      </c>
-      <c r="J12" s="16" t="s">
+        <v>2846.2</v>
+      </c>
+      <c r="J12" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K12" s="16" t="s">
-        <v>58</v>
+      <c r="K12" s="13" t="s">
+        <v>59</v>
       </c>
       <c r="L12" s="17">
         <v>2.05</v>
@@ -1336,38 +1333,38 @@
       <c r="O12" s="17">
         <v>3214.4</v>
       </c>
-      <c r="P12" s="13" t="s">
+      <c r="P12" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="Q12" s="13" t="s">
+      <c r="Q12" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="R12" s="17">
+      <c r="R12" s="15">
         <v>80</v>
       </c>
-      <c r="S12" s="18">
+      <c r="S12" s="16">
         <v>10</v>
       </c>
-      <c r="T12" s="17">
+      <c r="T12" s="15">
         <v>72</v>
       </c>
-      <c r="U12" s="17">
-        <v>2520</v>
+      <c r="U12" s="15">
+        <v>2880</v>
       </c>
       <c r="V12" s="13" t="s">
         <v>48</v>
       </c>
       <c r="W12" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="X12" s="16" t="s">
-        <v>49</v>
+        <v>60</v>
+      </c>
+      <c r="X12" s="18" t="s">
+        <v>61</v>
       </c>
       <c r="Y12" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z12" s="15">
-        <v>284.62</v>
+        <v>56</v>
+      </c>
+      <c r="Z12" s="17">
+        <v>3214.4</v>
       </c>
       <c r="AA12" s="14" t="s">
         <v>51</v>
@@ -1378,16 +1375,16 @@
         <v>4</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E13" s="13">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="F13" s="15">
         <v>2.1</v>
@@ -1399,12 +1396,12 @@
         <v>88.08240000000001</v>
       </c>
       <c r="I13" s="15">
-        <v>704.6592000000001</v>
-      </c>
-      <c r="J13" s="16" t="s">
+        <v>7046.592</v>
+      </c>
+      <c r="J13" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K13" s="16" t="s">
+      <c r="K13" s="13" t="s">
         <v>46</v>
       </c>
       <c r="L13" s="17">
@@ -1417,40 +1414,40 @@
         <v>71.06959999999999</v>
       </c>
       <c r="O13" s="17">
-        <v>5685.567999999999</v>
-      </c>
-      <c r="P13" s="13" t="s">
+        <v>5685.568</v>
+      </c>
+      <c r="P13" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="Q13" s="13" t="s">
+      <c r="Q13" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="R13" s="17">
+      <c r="R13" s="15">
         <v>70</v>
       </c>
-      <c r="S13" s="18">
+      <c r="S13" s="16">
         <v>7</v>
       </c>
-      <c r="T13" s="17">
+      <c r="T13" s="15">
         <v>65.09999999999999</v>
       </c>
-      <c r="U13" s="17">
-        <v>4557</v>
+      <c r="U13" s="15">
+        <v>5208</v>
       </c>
       <c r="V13" s="13" t="s">
         <v>55</v>
       </c>
       <c r="W13" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="X13" s="16" t="s">
-        <v>49</v>
+        <v>64</v>
+      </c>
+      <c r="X13" s="18" t="s">
+        <v>61</v>
       </c>
       <c r="Y13" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z13" s="15">
-        <v>704.6592000000001</v>
+        <v>56</v>
+      </c>
+      <c r="Z13" s="17">
+        <v>5685.568</v>
       </c>
       <c r="AA13" s="14" t="s">
         <v>51</v>
@@ -1461,16 +1458,16 @@
         <v>5</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E14" s="13">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F14" s="15">
         <v>1</v>
@@ -1482,31 +1479,31 @@
         <v>42.372</v>
       </c>
       <c r="I14" s="15">
-        <v>42.372</v>
-      </c>
-      <c r="J14" s="16" t="s">
+        <v>423.72</v>
+      </c>
+      <c r="J14" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K14" s="16" t="s">
+      <c r="K14" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="L14" s="17">
+      <c r="L14" s="15">
         <v>2</v>
       </c>
-      <c r="M14" s="18">
+      <c r="M14" s="16">
         <v>10</v>
       </c>
-      <c r="N14" s="17">
+      <c r="N14" s="15">
         <v>70.56</v>
       </c>
-      <c r="O14" s="17">
+      <c r="O14" s="15">
         <v>705.6</v>
       </c>
       <c r="P14" s="13" t="s">
         <v>54</v>
       </c>
       <c r="Q14" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="R14" s="17">
         <v>78</v>
@@ -1520,20 +1517,20 @@
       <c r="U14" s="17">
         <v>686.4</v>
       </c>
-      <c r="V14" s="13" t="s">
+      <c r="V14" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="W14" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="X14" s="16" t="s">
+      <c r="W14" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="X14" s="18" t="s">
         <v>49</v>
       </c>
       <c r="Y14" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z14" s="15">
-        <v>42.372</v>
+        <v>56</v>
+      </c>
+      <c r="Z14" s="17">
+        <v>686.4</v>
       </c>
       <c r="AA14" s="14" t="s">
         <v>51</v>
@@ -1544,16 +1541,16 @@
         <v>6</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E15" s="13">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F15" s="15">
         <v>0.4</v>
@@ -1565,24 +1562,24 @@
         <v>16.264</v>
       </c>
       <c r="I15" s="15">
-        <v>32.528</v>
-      </c>
-      <c r="J15" s="16" t="s">
+        <v>325.28</v>
+      </c>
+      <c r="J15" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="K15" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="L15" s="17">
+      <c r="K15" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="L15" s="15">
         <v>0.28</v>
       </c>
-      <c r="M15" s="18">
+      <c r="M15" s="16">
         <v>0</v>
       </c>
-      <c r="N15" s="17">
+      <c r="N15" s="15">
         <v>10.976</v>
       </c>
-      <c r="O15" s="17">
+      <c r="O15" s="15">
         <v>219.52</v>
       </c>
       <c r="P15" s="13" t="s">
@@ -1603,20 +1600,20 @@
       <c r="U15" s="17">
         <v>180</v>
       </c>
-      <c r="V15" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="W15" s="13" t="s">
+      <c r="V15" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="W15" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="X15" s="16" t="s">
+      <c r="X15" s="18" t="s">
         <v>49</v>
       </c>
       <c r="Y15" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="Z15" s="15">
-        <v>32.528</v>
+      <c r="Z15" s="17">
+        <v>180</v>
       </c>
       <c r="AA15" s="14" t="s">
         <v>51</v>
@@ -1627,16 +1624,16 @@
         <v>7</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E16" s="13">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F16" s="19" t="s">
         <v>51</v>
@@ -1656,49 +1653,49 @@
       <c r="K16" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="L16" s="17">
+      <c r="L16" s="15">
         <v>0.62</v>
       </c>
-      <c r="M16" s="18">
+      <c r="M16" s="16">
         <v>3</v>
       </c>
-      <c r="N16" s="17">
+      <c r="N16" s="15">
         <v>23.5749</v>
       </c>
-      <c r="O16" s="17">
-        <v>353.6235</v>
+      <c r="O16" s="15">
+        <v>471.4976</v>
       </c>
       <c r="P16" s="13" t="s">
         <v>45</v>
       </c>
       <c r="Q16" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="R16" s="15">
+        <v>60</v>
+      </c>
+      <c r="R16" s="17">
         <v>20</v>
       </c>
-      <c r="S16" s="16">
+      <c r="S16" s="18">
         <v>4</v>
       </c>
-      <c r="T16" s="15">
+      <c r="T16" s="17">
         <v>19.2</v>
       </c>
-      <c r="U16" s="15">
+      <c r="U16" s="17">
         <v>384</v>
       </c>
-      <c r="V16" s="16" t="s">
+      <c r="V16" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="W16" s="16" t="s">
+      <c r="W16" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="X16" s="16" t="s">
-        <v>73</v>
+      <c r="X16" s="18" t="s">
+        <v>49</v>
       </c>
       <c r="Y16" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z16" s="15">
+        <v>50</v>
+      </c>
+      <c r="Z16" s="17">
         <v>384</v>
       </c>
       <c r="AA16" s="14" t="s">
@@ -1719,7 +1716,7 @@
         <v>44</v>
       </c>
       <c r="E17" s="13">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F17" s="19" t="s">
         <v>51</v>
@@ -1749,13 +1746,13 @@
         <v>57.722</v>
       </c>
       <c r="O17" s="15">
-        <v>2597.49</v>
-      </c>
-      <c r="P17" s="16" t="s">
+        <v>2886.1</v>
+      </c>
+      <c r="P17" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="Q17" s="16" t="s">
-        <v>59</v>
+      <c r="Q17" s="13" t="s">
+        <v>60</v>
       </c>
       <c r="R17" s="17">
         <v>60</v>
@@ -1769,20 +1766,20 @@
       <c r="U17" s="17">
         <v>2760</v>
       </c>
-      <c r="V17" s="13" t="s">
+      <c r="V17" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="W17" s="13" t="s">
+      <c r="W17" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="X17" s="16" t="s">
-        <v>76</v>
+      <c r="X17" s="18" t="s">
+        <v>49</v>
       </c>
       <c r="Y17" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="Z17" s="15">
-        <v>2597.49</v>
+      <c r="Z17" s="17">
+        <v>2760</v>
       </c>
       <c r="AA17" s="14" t="s">
         <v>51</v>
@@ -1793,16 +1790,16 @@
         <v>9</v>
       </c>
       <c r="B18" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" s="14" t="s">
         <v>77</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>78</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E18" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F18" s="19" t="s">
         <v>51</v>
@@ -1832,13 +1829,13 @@
         <v>94.08</v>
       </c>
       <c r="O18" s="15">
-        <v>376.32</v>
-      </c>
-      <c r="P18" s="16" t="s">
+        <v>470.4</v>
+      </c>
+      <c r="P18" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="Q18" s="16" t="s">
-        <v>69</v>
+      <c r="Q18" s="13" t="s">
+        <v>70</v>
       </c>
       <c r="R18" s="17">
         <v>90</v>
@@ -1852,20 +1849,20 @@
       <c r="U18" s="17">
         <v>405</v>
       </c>
-      <c r="V18" s="13" t="s">
+      <c r="V18" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="W18" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="X18" s="16" t="s">
-        <v>76</v>
+      <c r="W18" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="X18" s="18" t="s">
+        <v>49</v>
       </c>
       <c r="Y18" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="Z18" s="15">
-        <v>376.32</v>
+      <c r="Z18" s="17">
+        <v>405</v>
       </c>
       <c r="AA18" s="14" t="s">
         <v>51</v>
@@ -1876,10 +1873,10 @@
         <v>10</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="14" t="s">
         <v>80</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>81</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>44</v>
@@ -1905,16 +1902,16 @@
       <c r="K19" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="L19" s="17">
+      <c r="L19" s="15">
         <v>0.22</v>
       </c>
-      <c r="M19" s="18">
+      <c r="M19" s="16">
         <v>0</v>
       </c>
-      <c r="N19" s="17">
+      <c r="N19" s="15">
         <v>8.624000000000001</v>
       </c>
-      <c r="O19" s="17">
+      <c r="O19" s="15">
         <v>258.72</v>
       </c>
       <c r="P19" s="13" t="s">
@@ -1923,31 +1920,31 @@
       <c r="Q19" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="R19" s="15">
+      <c r="R19" s="17">
         <v>10</v>
       </c>
-      <c r="S19" s="16">
+      <c r="S19" s="18">
         <v>10</v>
       </c>
-      <c r="T19" s="15">
+      <c r="T19" s="17">
         <v>9</v>
       </c>
-      <c r="U19" s="15">
+      <c r="U19" s="17">
         <v>270</v>
       </c>
-      <c r="V19" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="W19" s="16" t="s">
+      <c r="V19" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="W19" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="X19" s="16" t="s">
-        <v>73</v>
+      <c r="X19" s="18" t="s">
+        <v>49</v>
       </c>
       <c r="Y19" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z19" s="15">
+        <v>56</v>
+      </c>
+      <c r="Z19" s="17">
         <v>270</v>
       </c>
       <c r="AA19" s="14" t="s">
@@ -1955,26 +1952,26 @@
       </c>
     </row>
     <row r="21" spans="1:27">
-      <c r="A21" s="16"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D21" s="21"/>
       <c r="E21" s="20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G21" s="22"/>
       <c r="H21" s="20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K21" s="19"/>
       <c r="L21" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:27">
       <c r="A24" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1982,7 +1979,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
@@ -1990,7 +1987,7 @@
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
       <c r="M24" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
@@ -1998,7 +1995,7 @@
       <c r="Q24" s="3"/>
       <c r="R24" s="3"/>
       <c r="S24" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
@@ -2008,7 +2005,7 @@
     </row>
     <row r="25" spans="1:27">
       <c r="A25" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -2016,16 +2013,16 @@
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
       <c r="G25" s="23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H25" s="23" t="s">
         <v>25</v>
       </c>
       <c r="I25" s="23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N25" s="5"/>
       <c r="O25" s="5"/>
@@ -2033,7 +2030,7 @@
       <c r="Q25" s="5"/>
       <c r="R25" s="5"/>
       <c r="S25" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="T25" s="5"/>
       <c r="U25" s="5"/>
@@ -2049,7 +2046,7 @@
       <c r="E26" s="5"/>
       <c r="F26" s="5"/>
       <c r="G26" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
@@ -2154,10 +2151,10 @@
     </row>
     <row r="32" spans="1:27">
       <c r="A32" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="K32" s="20" t="s">
         <v>96</v>
-      </c>
-      <c r="K32" s="20" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
talepler tekliflere teklifler siparişlere bağlandı. Son aşama henüz kontrol edilmedi.
</commit_message>
<xml_diff>
--- a/backend/app/temp/mukayese_raporu.xlsx
+++ b/backend/app/temp/mukayese_raporu.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="130">
   <si>
     <t>TEKLİF KARŞILAŞTIRMA RAPORU</t>
   </si>
@@ -46,7 +46,7 @@
     <t>En Avantajlı Firma Dağılımı</t>
   </si>
   <si>
-    <t>AYDIN KIRTASİYE LTD. ŞTİ.: 12  Teklif Kardelen Ofis: 2</t>
+    <t>Teklif Zirve Tedarik: 14</t>
   </si>
   <si>
     <t>Para Birimi</t>
@@ -64,7 +64,7 @@
     <t>05.05.2026</t>
   </si>
   <si>
-    <t>16:10</t>
+    <t>21:39</t>
   </si>
   <si>
     <t>Bilgilendirme</t>
@@ -121,9 +121,6 @@
     <t>BETA KIRTASİYE PAZARLAMA</t>
   </si>
   <si>
-    <t>FIRMA 6</t>
-  </si>
-  <si>
     <t>MAVİ OFİS TEDARİK A.Ş.</t>
   </si>
   <si>
@@ -133,6 +130,9 @@
     <t>TEKLIF KARDELEN OFIS</t>
   </si>
   <si>
+    <t>TEKLIF ZIRVE TEDARIK</t>
+  </si>
+  <si>
     <t>KARAR / ÖNERİ</t>
   </si>
   <si>
@@ -142,7 +142,7 @@
     <t>Karar Nedeni</t>
   </si>
   <si>
-    <t>En Avantajlı Net Tutar (TRY)</t>
+    <t>En Avantajlı Değerlendirilmiş Maliyet (TRY)</t>
   </si>
   <si>
     <t>Not</t>
@@ -169,34 +169,37 @@
     <t>Termin 5 iş günü</t>
   </si>
   <si>
+    <t>Vade 60 gün</t>
+  </si>
+  <si>
+    <t>Termin 7 iş günü</t>
+  </si>
+  <si>
+    <t>Vade 90 gün</t>
+  </si>
+  <si>
+    <t>Termin 10 iş günü</t>
+  </si>
+  <si>
+    <t>30 gün</t>
+  </si>
+  <si>
+    <t>14 iş günü</t>
+  </si>
+  <si>
     <t>75 gün</t>
   </si>
   <si>
     <t>4 iş günü</t>
   </si>
   <si>
-    <t>Vade 60 gün</t>
-  </si>
-  <si>
-    <t>Termin 7 iş günü</t>
-  </si>
-  <si>
-    <t>Vade 90 gün</t>
-  </si>
-  <si>
-    <t>Termin 10 iş günü</t>
-  </si>
-  <si>
-    <t>30 gün</t>
-  </si>
-  <si>
-    <t>14 iş günü</t>
-  </si>
-  <si>
-    <t>Vade avantajlı</t>
-  </si>
-  <si>
-    <t>%5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 144.06 TRY</t>
+    <t>Teklif Zirve Tedarik</t>
+  </si>
+  <si>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 7,302.10 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 675.19 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>A102</t>
@@ -205,7 +208,10 @@
     <t>SİLGİ BÜYÜK</t>
   </si>
   <si>
-    <t>%3 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 69.06 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 2,439.25 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%4 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 225.55 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>A103</t>
@@ -214,7 +220,10 @@
     <t>DEFTER A4</t>
   </si>
   <si>
-    <t>%5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 105.41 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 5,974.50 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 552.44 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>a004</t>
@@ -223,7 +232,10 @@
     <t>PERGEL</t>
   </si>
   <si>
-    <t>%5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 137.03 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 7,997.60 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 739.50 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>a005</t>
@@ -232,7 +244,10 @@
     <t>CETVEL</t>
   </si>
   <si>
-    <t>%5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 29.52 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 1,310.40 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 121.17 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>PRD-0001</t>
@@ -241,7 +256,10 @@
     <t>PİLOT KALEM</t>
   </si>
   <si>
-    <t>*Otomatik kod | %5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 34.79 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 1,249.20 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>*Otomatik kod | %6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 115.51 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>A104</t>
@@ -250,7 +268,10 @@
     <t>DOSYA KLASÖR</t>
   </si>
   <si>
-    <t>%5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 42.16 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 1,642.20 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 151.85 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>A105</t>
@@ -259,10 +280,10 @@
     <t>ZIMBA MAKİNESİ</t>
   </si>
   <si>
-    <t>Teklif Kardelen Ofis</t>
-  </si>
-  <si>
-    <t>%12 iskonto | 30 gün vade | 14 gün termin | Vade avantajı: 198.41 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 6,548.80 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 605.54 TRY | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>a001</t>
@@ -271,7 +292,10 @@
     <t>silgi</t>
   </si>
   <si>
-    <t>%5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 19.33 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 874.50 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 80.86 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>a002</t>
@@ -280,7 +304,10 @@
     <t>defter</t>
   </si>
   <si>
-    <t>%10 iskonto | 30 gün vade | 14 gün termin | Vade avantajı: 116.52 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 3,841.20 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%4 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 355.18 TRY | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>a003</t>
@@ -289,7 +316,10 @@
     <t>kalem tıraş</t>
   </si>
   <si>
-    <t>%3 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 57.40 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 2,555.20 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%4 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 236.27 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>a006</t>
@@ -298,7 +328,10 @@
     <t>kalem</t>
   </si>
   <si>
-    <t>%3 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 1.79 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 61.70 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%4 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 5.71 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>AA001</t>
@@ -307,7 +340,10 @@
     <t>kurşun kalem</t>
   </si>
   <si>
-    <t>%5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 8.78 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 450.50 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 41.66 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>PRD-0002</t>
@@ -316,7 +352,10 @@
     <t>uçlu kalem</t>
   </si>
   <si>
-    <t>*Otomatik kod | %5 iskonto | 30 gün vade | 3 gün termin | Vade avantajı: 36.89 TRY</t>
+    <t>Teklif Zirve Tedarik önerildi; bütçe, vade ve termin kriterlerini sağlıyor. Net toplam: 1,483.30 TRY, vade: 75 gün, termin: 4 gün.</t>
+  </si>
+  <si>
+    <t>*Otomatik kod | %6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 137.15 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 60 gün, teklif 30 gün; Kriter dışı: maksimum termin 6 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: maksimum termin 6 gün, teklif 7 gün; Elendi: Maksimum termin şartını aşıyor (7 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 6 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 60 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>Önerilen / en avantajlı teklif</t>
@@ -378,18 +417,19 @@
     <t>Rapor Oluşturan: Sistem</t>
   </si>
   <si>
-    <t>Rapor No: RPR-20260505-1610</t>
+    <t>Rapor No: RPR-20260505-2139</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0.00"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="#,##0.00 ₺"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,6 +488,13 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFB91C1C"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -529,13 +576,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCFE8C8"/>
+        <fgColor rgb="FFF5B7B1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5B7B1"/>
+        <fgColor rgb="FFCFE8C8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -630,22 +677,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1360,143 +1407,143 @@
       <c r="K10" s="18">
         <v>3750.9384</v>
       </c>
-      <c r="L10" s="19" t="s">
+      <c r="L10" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M10" s="19" t="s">
+      <c r="M10" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N10" s="20">
+      <c r="N10" s="18">
         <v>17.86</v>
       </c>
-      <c r="O10" s="21">
+      <c r="O10" s="19">
         <v>3</v>
       </c>
-      <c r="P10" s="20">
+      <c r="P10" s="18">
         <v>17.32</v>
       </c>
-      <c r="Q10" s="20">
+      <c r="Q10" s="18">
         <v>7101.2</v>
       </c>
-      <c r="R10" s="20">
+      <c r="R10" s="18">
         <v>7101.2</v>
       </c>
-      <c r="S10" s="20">
+      <c r="S10" s="18">
         <v>6707.2293</v>
       </c>
-      <c r="T10" s="16" t="s">
+      <c r="T10" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U10" s="16" t="s">
+      <c r="U10" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V10" s="20">
+      <c r="V10" s="18">
+        <v>17.13</v>
+      </c>
+      <c r="W10" s="19">
+        <v>8</v>
+      </c>
+      <c r="X10" s="18">
+        <v>15.7596</v>
+      </c>
+      <c r="Y10" s="18">
+        <v>6461.436</v>
+      </c>
+      <c r="Z10" s="18">
+        <v>6461.436</v>
+      </c>
+      <c r="AA10" s="18">
+        <v>5983.4668</v>
+      </c>
+      <c r="AB10" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC10" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD10" s="18">
+        <v>19.68</v>
+      </c>
+      <c r="AE10" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF10" s="18">
+        <v>17.71</v>
+      </c>
+      <c r="AG10" s="18">
+        <v>7261.1</v>
+      </c>
+      <c r="AH10" s="18">
+        <v>7261.1</v>
+      </c>
+      <c r="AI10" s="18">
+        <v>6455.4163</v>
+      </c>
+      <c r="AJ10" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK10" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL10" s="18">
+        <v>16.58</v>
+      </c>
+      <c r="AM10" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN10" s="18">
+        <v>14.59</v>
+      </c>
+      <c r="AO10" s="18">
+        <v>5981.9</v>
+      </c>
+      <c r="AP10" s="18">
+        <v>5981.9</v>
+      </c>
+      <c r="AQ10" s="18">
+        <v>5760.6516</v>
+      </c>
+      <c r="AR10" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS10" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT10" s="21">
         <v>18.95</v>
       </c>
-      <c r="W10" s="21">
+      <c r="AU10" s="22">
         <v>6</v>
       </c>
-      <c r="X10" s="20">
+      <c r="AV10" s="21">
         <v>17.81</v>
       </c>
-      <c r="Y10" s="20">
+      <c r="AW10" s="21">
         <v>7302.1</v>
       </c>
-      <c r="Z10" s="20">
+      <c r="AX10" s="21">
         <v>7302.1</v>
       </c>
-      <c r="AA10" s="20">
+      <c r="AY10" s="21">
         <v>6626.9058</v>
       </c>
-      <c r="AB10" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC10" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD10" s="20">
-        <v>17.13</v>
-      </c>
-      <c r="AE10" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF10" s="20">
-        <v>15.7596</v>
-      </c>
-      <c r="AG10" s="20">
-        <v>6461.436</v>
-      </c>
-      <c r="AH10" s="20">
-        <v>6461.436</v>
-      </c>
-      <c r="AI10" s="20">
-        <v>5983.4668</v>
-      </c>
-      <c r="AJ10" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK10" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL10" s="20">
-        <v>19.68</v>
-      </c>
-      <c r="AM10" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN10" s="20">
-        <v>17.71</v>
-      </c>
-      <c r="AO10" s="20">
-        <v>7261.1</v>
-      </c>
-      <c r="AP10" s="20">
-        <v>7261.1</v>
-      </c>
-      <c r="AQ10" s="20">
-        <v>6455.4163</v>
-      </c>
-      <c r="AR10" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS10" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT10" s="20">
-        <v>16.58</v>
-      </c>
-      <c r="AU10" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV10" s="20">
-        <v>14.59</v>
-      </c>
-      <c r="AW10" s="20">
-        <v>5981.9</v>
-      </c>
-      <c r="AX10" s="20">
-        <v>5981.9</v>
-      </c>
-      <c r="AY10" s="20">
-        <v>5760.6516</v>
-      </c>
-      <c r="AZ10" s="16" t="s">
+      <c r="AZ10" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA10" s="16" t="s">
+      <c r="BA10" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB10" s="19" t="s">
-        <v>25</v>
+      <c r="BB10" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC10" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD10" s="18">
-        <v>3895</v>
+        <v>60</v>
+      </c>
+      <c r="BD10" s="21">
+        <v>6626.9058</v>
       </c>
       <c r="BE10" s="17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:57">
@@ -1504,10 +1551,10 @@
         <v>2</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>46</v>
@@ -1533,143 +1580,143 @@
       <c r="K11" s="18">
         <v>1798.1873</v>
       </c>
-      <c r="L11" s="19" t="s">
+      <c r="L11" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M11" s="19" t="s">
+      <c r="M11" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N11" s="20">
+      <c r="N11" s="18">
         <v>8.699999999999999</v>
       </c>
-      <c r="O11" s="21">
+      <c r="O11" s="19">
         <v>1</v>
       </c>
-      <c r="P11" s="20">
+      <c r="P11" s="18">
         <v>8.609999999999999</v>
       </c>
-      <c r="Q11" s="20">
+      <c r="Q11" s="18">
         <v>2367.75</v>
       </c>
-      <c r="R11" s="20">
+      <c r="R11" s="18">
         <v>2367.75</v>
       </c>
-      <c r="S11" s="20">
+      <c r="S11" s="18">
         <v>2236.3885</v>
       </c>
-      <c r="T11" s="16" t="s">
+      <c r="T11" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U11" s="16" t="s">
+      <c r="U11" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V11" s="20">
+      <c r="V11" s="18">
+        <v>8.35</v>
+      </c>
+      <c r="W11" s="19">
+        <v>6</v>
+      </c>
+      <c r="X11" s="18">
+        <v>7.849</v>
+      </c>
+      <c r="Y11" s="18">
+        <v>2158.475</v>
+      </c>
+      <c r="Z11" s="18">
+        <v>2158.475</v>
+      </c>
+      <c r="AA11" s="18">
+        <v>1998.807</v>
+      </c>
+      <c r="AB11" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC11" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD11" s="18">
+        <v>9.59</v>
+      </c>
+      <c r="AE11" s="19">
+        <v>8</v>
+      </c>
+      <c r="AF11" s="18">
+        <v>8.82</v>
+      </c>
+      <c r="AG11" s="18">
+        <v>2425.5</v>
+      </c>
+      <c r="AH11" s="18">
+        <v>2425.5</v>
+      </c>
+      <c r="AI11" s="18">
+        <v>2156.3692</v>
+      </c>
+      <c r="AJ11" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK11" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL11" s="18">
+        <v>8.08</v>
+      </c>
+      <c r="AM11" s="19">
+        <v>10</v>
+      </c>
+      <c r="AN11" s="18">
+        <v>7.27</v>
+      </c>
+      <c r="AO11" s="18">
+        <v>1999.25</v>
+      </c>
+      <c r="AP11" s="18">
+        <v>1999.25</v>
+      </c>
+      <c r="AQ11" s="18">
+        <v>1925.3051</v>
+      </c>
+      <c r="AR11" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS11" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT11" s="21">
         <v>9.24</v>
       </c>
-      <c r="W11" s="21">
+      <c r="AU11" s="22">
         <v>4</v>
       </c>
-      <c r="X11" s="20">
+      <c r="AV11" s="21">
         <v>8.869999999999999</v>
       </c>
-      <c r="Y11" s="20">
+      <c r="AW11" s="21">
         <v>2439.25</v>
       </c>
-      <c r="Z11" s="20">
+      <c r="AX11" s="21">
         <v>2439.25</v>
       </c>
-      <c r="AA11" s="20">
+      <c r="AY11" s="21">
         <v>2213.7029</v>
       </c>
-      <c r="AB11" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC11" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD11" s="20">
-        <v>8.35</v>
-      </c>
-      <c r="AE11" s="21">
-        <v>6</v>
-      </c>
-      <c r="AF11" s="20">
-        <v>7.849</v>
-      </c>
-      <c r="AG11" s="20">
-        <v>2158.475</v>
-      </c>
-      <c r="AH11" s="20">
-        <v>2158.475</v>
-      </c>
-      <c r="AI11" s="20">
-        <v>1998.807</v>
-      </c>
-      <c r="AJ11" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK11" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL11" s="20">
-        <v>9.59</v>
-      </c>
-      <c r="AM11" s="21">
-        <v>8</v>
-      </c>
-      <c r="AN11" s="20">
-        <v>8.82</v>
-      </c>
-      <c r="AO11" s="20">
-        <v>2425.5</v>
-      </c>
-      <c r="AP11" s="20">
-        <v>2425.5</v>
-      </c>
-      <c r="AQ11" s="20">
-        <v>2156.3692</v>
-      </c>
-      <c r="AR11" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS11" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT11" s="20">
-        <v>8.08</v>
-      </c>
-      <c r="AU11" s="21">
-        <v>10</v>
-      </c>
-      <c r="AV11" s="20">
-        <v>7.27</v>
-      </c>
-      <c r="AW11" s="20">
-        <v>1999.25</v>
-      </c>
-      <c r="AX11" s="20">
-        <v>1999.25</v>
-      </c>
-      <c r="AY11" s="20">
-        <v>1925.3051</v>
-      </c>
-      <c r="AZ11" s="16" t="s">
+      <c r="AZ11" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA11" s="16" t="s">
+      <c r="BA11" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB11" s="19" t="s">
-        <v>25</v>
+      <c r="BB11" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC11" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD11" s="18">
-        <v>1867.25</v>
+        <v>64</v>
+      </c>
+      <c r="BD11" s="21">
+        <v>2213.7029</v>
       </c>
       <c r="BE11" s="17" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:57">
@@ -1677,10 +1724,10 @@
         <v>3</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D12" s="16" t="s">
         <v>46</v>
@@ -1706,143 +1753,143 @@
       <c r="K12" s="18">
         <v>2744.589</v>
       </c>
-      <c r="L12" s="19" t="s">
+      <c r="L12" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M12" s="19" t="s">
+      <c r="M12" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N12" s="20">
+      <c r="N12" s="18">
         <v>39.93</v>
       </c>
-      <c r="O12" s="21">
+      <c r="O12" s="19">
         <v>3</v>
       </c>
-      <c r="P12" s="20">
+      <c r="P12" s="18">
         <v>38.73</v>
       </c>
-      <c r="Q12" s="20">
+      <c r="Q12" s="18">
         <v>5809.5</v>
       </c>
-      <c r="R12" s="20">
+      <c r="R12" s="18">
         <v>5809.5</v>
       </c>
-      <c r="S12" s="20">
+      <c r="S12" s="18">
         <v>5487.1921</v>
       </c>
-      <c r="T12" s="16" t="s">
+      <c r="T12" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U12" s="16" t="s">
+      <c r="U12" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V12" s="20">
+      <c r="V12" s="18">
+        <v>38.3</v>
+      </c>
+      <c r="W12" s="19">
+        <v>8</v>
+      </c>
+      <c r="X12" s="18">
+        <v>35.236</v>
+      </c>
+      <c r="Y12" s="18">
+        <v>5285.4</v>
+      </c>
+      <c r="Z12" s="18">
+        <v>5285.4</v>
+      </c>
+      <c r="AA12" s="18">
+        <v>4894.4252</v>
+      </c>
+      <c r="AB12" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC12" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD12" s="18">
+        <v>44</v>
+      </c>
+      <c r="AE12" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF12" s="18">
+        <v>39.6</v>
+      </c>
+      <c r="AG12" s="18">
+        <v>5940</v>
+      </c>
+      <c r="AH12" s="18">
+        <v>5940</v>
+      </c>
+      <c r="AI12" s="18">
+        <v>5280.9041</v>
+      </c>
+      <c r="AJ12" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK12" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL12" s="18">
+        <v>37.07</v>
+      </c>
+      <c r="AM12" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN12" s="18">
+        <v>32.62</v>
+      </c>
+      <c r="AO12" s="18">
+        <v>4893</v>
+      </c>
+      <c r="AP12" s="18">
+        <v>4893</v>
+      </c>
+      <c r="AQ12" s="18">
+        <v>4712.026</v>
+      </c>
+      <c r="AR12" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS12" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT12" s="21">
         <v>42.37</v>
       </c>
-      <c r="W12" s="21">
+      <c r="AU12" s="22">
         <v>6</v>
       </c>
-      <c r="X12" s="20">
+      <c r="AV12" s="21">
         <v>39.83</v>
       </c>
-      <c r="Y12" s="20">
+      <c r="AW12" s="21">
         <v>5974.5</v>
       </c>
-      <c r="Z12" s="20">
+      <c r="AX12" s="21">
         <v>5974.5</v>
       </c>
-      <c r="AA12" s="20">
+      <c r="AY12" s="21">
         <v>5422.0634</v>
       </c>
-      <c r="AB12" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC12" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD12" s="20">
-        <v>38.3</v>
-      </c>
-      <c r="AE12" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF12" s="20">
-        <v>35.236</v>
-      </c>
-      <c r="AG12" s="20">
-        <v>5285.4</v>
-      </c>
-      <c r="AH12" s="20">
-        <v>5285.4</v>
-      </c>
-      <c r="AI12" s="20">
-        <v>4894.4252</v>
-      </c>
-      <c r="AJ12" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK12" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL12" s="20">
-        <v>44</v>
-      </c>
-      <c r="AM12" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN12" s="20">
-        <v>39.6</v>
-      </c>
-      <c r="AO12" s="20">
-        <v>5940</v>
-      </c>
-      <c r="AP12" s="20">
-        <v>5940</v>
-      </c>
-      <c r="AQ12" s="20">
-        <v>5280.9041</v>
-      </c>
-      <c r="AR12" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS12" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT12" s="20">
-        <v>37.07</v>
-      </c>
-      <c r="AU12" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV12" s="20">
-        <v>32.62</v>
-      </c>
-      <c r="AW12" s="20">
-        <v>4893</v>
-      </c>
-      <c r="AX12" s="20">
-        <v>4893</v>
-      </c>
-      <c r="AY12" s="20">
-        <v>4712.026</v>
-      </c>
-      <c r="AZ12" s="16" t="s">
+      <c r="AZ12" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA12" s="16" t="s">
+      <c r="BA12" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB12" s="19" t="s">
-        <v>25</v>
+      <c r="BB12" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC12" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD12" s="18">
-        <v>2850</v>
+        <v>68</v>
+      </c>
+      <c r="BD12" s="21">
+        <v>5422.0634</v>
       </c>
       <c r="BE12" s="17" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:57">
@@ -1850,10 +1897,10 @@
         <v>4</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>46</v>
@@ -1879,143 +1926,143 @@
       <c r="K13" s="18">
         <v>3567.9658</v>
       </c>
-      <c r="L13" s="19" t="s">
+      <c r="L13" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M13" s="19" t="s">
+      <c r="M13" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N13" s="20">
+      <c r="N13" s="18">
         <v>30.84</v>
       </c>
-      <c r="O13" s="21">
+      <c r="O13" s="19">
         <v>3</v>
       </c>
-      <c r="P13" s="20">
+      <c r="P13" s="18">
         <v>29.91</v>
       </c>
-      <c r="Q13" s="20">
+      <c r="Q13" s="18">
         <v>7776.6</v>
       </c>
-      <c r="R13" s="20">
+      <c r="R13" s="18">
         <v>7776.6</v>
       </c>
-      <c r="S13" s="20">
+      <c r="S13" s="18">
         <v>7345.1585</v>
       </c>
-      <c r="T13" s="16" t="s">
+      <c r="T13" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U13" s="16" t="s">
+      <c r="U13" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V13" s="20">
+      <c r="V13" s="18">
+        <v>29.58</v>
+      </c>
+      <c r="W13" s="19">
+        <v>8</v>
+      </c>
+      <c r="X13" s="18">
+        <v>27.2136</v>
+      </c>
+      <c r="Y13" s="18">
+        <v>7075.536</v>
+      </c>
+      <c r="Z13" s="18">
+        <v>7075.536</v>
+      </c>
+      <c r="AA13" s="18">
+        <v>6552.1402</v>
+      </c>
+      <c r="AB13" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC13" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD13" s="18">
+        <v>33.98</v>
+      </c>
+      <c r="AE13" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF13" s="18">
+        <v>30.58</v>
+      </c>
+      <c r="AG13" s="18">
+        <v>7950.8</v>
+      </c>
+      <c r="AH13" s="18">
+        <v>7950.8</v>
+      </c>
+      <c r="AI13" s="18">
+        <v>7068.5879</v>
+      </c>
+      <c r="AJ13" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK13" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL13" s="18">
+        <v>28.63</v>
+      </c>
+      <c r="AM13" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN13" s="18">
+        <v>25.19</v>
+      </c>
+      <c r="AO13" s="18">
+        <v>6549.4</v>
+      </c>
+      <c r="AP13" s="18">
+        <v>6549.4</v>
+      </c>
+      <c r="AQ13" s="18">
+        <v>6307.1619</v>
+      </c>
+      <c r="AR13" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS13" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT13" s="21">
         <v>32.72</v>
       </c>
-      <c r="W13" s="21">
+      <c r="AU13" s="22">
         <v>6</v>
       </c>
-      <c r="X13" s="20">
+      <c r="AV13" s="21">
         <v>30.76</v>
       </c>
-      <c r="Y13" s="20">
+      <c r="AW13" s="21">
         <v>7997.6</v>
       </c>
-      <c r="Z13" s="20">
+      <c r="AX13" s="21">
         <v>7997.6</v>
       </c>
-      <c r="AA13" s="20">
+      <c r="AY13" s="21">
         <v>7258.0959</v>
       </c>
-      <c r="AB13" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC13" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD13" s="20">
-        <v>29.58</v>
-      </c>
-      <c r="AE13" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF13" s="20">
-        <v>27.2136</v>
-      </c>
-      <c r="AG13" s="20">
-        <v>7075.536</v>
-      </c>
-      <c r="AH13" s="20">
-        <v>7075.536</v>
-      </c>
-      <c r="AI13" s="20">
-        <v>6552.1402</v>
-      </c>
-      <c r="AJ13" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK13" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL13" s="20">
-        <v>33.98</v>
-      </c>
-      <c r="AM13" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN13" s="20">
-        <v>30.58</v>
-      </c>
-      <c r="AO13" s="20">
-        <v>7950.8</v>
-      </c>
-      <c r="AP13" s="20">
-        <v>7950.8</v>
-      </c>
-      <c r="AQ13" s="20">
-        <v>7068.5879</v>
-      </c>
-      <c r="AR13" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS13" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT13" s="20">
-        <v>28.63</v>
-      </c>
-      <c r="AU13" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV13" s="20">
-        <v>25.19</v>
-      </c>
-      <c r="AW13" s="20">
-        <v>6549.4</v>
-      </c>
-      <c r="AX13" s="20">
-        <v>6549.4</v>
-      </c>
-      <c r="AY13" s="20">
-        <v>6307.1619</v>
-      </c>
-      <c r="AZ13" s="16" t="s">
+      <c r="AZ13" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA13" s="16" t="s">
+      <c r="BA13" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB13" s="19" t="s">
-        <v>25</v>
+      <c r="BB13" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC13" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD13" s="18">
-        <v>3705</v>
+        <v>72</v>
+      </c>
+      <c r="BD13" s="21">
+        <v>7258.0959</v>
       </c>
       <c r="BE13" s="17" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:57">
@@ -2023,10 +2070,10 @@
         <v>5</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>46</v>
@@ -2052,143 +2099,143 @@
       <c r="K14" s="18">
         <v>768.4849</v>
       </c>
-      <c r="L14" s="19" t="s">
+      <c r="L14" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M14" s="19" t="s">
+      <c r="M14" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N14" s="20">
+      <c r="N14" s="18">
         <v>6.26</v>
       </c>
-      <c r="O14" s="21">
+      <c r="O14" s="19">
         <v>3</v>
       </c>
-      <c r="P14" s="20">
+      <c r="P14" s="18">
         <v>6.07</v>
       </c>
-      <c r="Q14" s="20">
+      <c r="Q14" s="18">
         <v>1274.7</v>
       </c>
-      <c r="R14" s="20">
+      <c r="R14" s="18">
         <v>1274.7</v>
       </c>
-      <c r="S14" s="20">
+      <c r="S14" s="18">
         <v>1203.9803</v>
       </c>
-      <c r="T14" s="16" t="s">
+      <c r="T14" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U14" s="16" t="s">
+      <c r="U14" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V14" s="20">
+      <c r="V14" s="18">
+        <v>6</v>
+      </c>
+      <c r="W14" s="19">
+        <v>8</v>
+      </c>
+      <c r="X14" s="18">
+        <v>5.52</v>
+      </c>
+      <c r="Y14" s="18">
+        <v>1159.2</v>
+      </c>
+      <c r="Z14" s="18">
+        <v>1159.2</v>
+      </c>
+      <c r="AA14" s="18">
+        <v>1073.451</v>
+      </c>
+      <c r="AB14" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC14" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD14" s="18">
+        <v>6.9</v>
+      </c>
+      <c r="AE14" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF14" s="18">
+        <v>6.21</v>
+      </c>
+      <c r="AG14" s="18">
+        <v>1304.1</v>
+      </c>
+      <c r="AH14" s="18">
+        <v>1304.1</v>
+      </c>
+      <c r="AI14" s="18">
+        <v>1159.3985</v>
+      </c>
+      <c r="AJ14" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK14" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL14" s="18">
+        <v>5.81</v>
+      </c>
+      <c r="AM14" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN14" s="18">
+        <v>5.11</v>
+      </c>
+      <c r="AO14" s="18">
+        <v>1073.1</v>
+      </c>
+      <c r="AP14" s="18">
+        <v>1073.1</v>
+      </c>
+      <c r="AQ14" s="18">
+        <v>1033.41</v>
+      </c>
+      <c r="AR14" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS14" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT14" s="21">
         <v>6.64</v>
       </c>
-      <c r="W14" s="21">
+      <c r="AU14" s="22">
         <v>6</v>
       </c>
-      <c r="X14" s="20">
+      <c r="AV14" s="21">
         <v>6.24</v>
       </c>
-      <c r="Y14" s="20">
+      <c r="AW14" s="21">
         <v>1310.4</v>
       </c>
-      <c r="Z14" s="20">
+      <c r="AX14" s="21">
         <v>1310.4</v>
       </c>
-      <c r="AA14" s="20">
+      <c r="AY14" s="21">
         <v>1189.2329</v>
       </c>
-      <c r="AB14" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC14" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD14" s="20">
-        <v>6</v>
-      </c>
-      <c r="AE14" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF14" s="20">
-        <v>5.52</v>
-      </c>
-      <c r="AG14" s="20">
-        <v>1159.2</v>
-      </c>
-      <c r="AH14" s="20">
-        <v>1159.2</v>
-      </c>
-      <c r="AI14" s="20">
-        <v>1073.451</v>
-      </c>
-      <c r="AJ14" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK14" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL14" s="20">
-        <v>6.9</v>
-      </c>
-      <c r="AM14" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN14" s="20">
-        <v>6.21</v>
-      </c>
-      <c r="AO14" s="20">
-        <v>1304.1</v>
-      </c>
-      <c r="AP14" s="20">
-        <v>1304.1</v>
-      </c>
-      <c r="AQ14" s="20">
-        <v>1159.3985</v>
-      </c>
-      <c r="AR14" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS14" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT14" s="20">
-        <v>5.81</v>
-      </c>
-      <c r="AU14" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV14" s="20">
-        <v>5.11</v>
-      </c>
-      <c r="AW14" s="20">
-        <v>1073.1</v>
-      </c>
-      <c r="AX14" s="20">
-        <v>1073.1</v>
-      </c>
-      <c r="AY14" s="20">
-        <v>1033.41</v>
-      </c>
-      <c r="AZ14" s="16" t="s">
+      <c r="AZ14" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA14" s="16" t="s">
+      <c r="BA14" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB14" s="19" t="s">
-        <v>25</v>
+      <c r="BB14" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC14" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD14" s="18">
-        <v>798</v>
+        <v>76</v>
+      </c>
+      <c r="BD14" s="21">
+        <v>1189.2329</v>
       </c>
       <c r="BE14" s="17" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:57">
@@ -2196,10 +2243,10 @@
         <v>6</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>46</v>
@@ -2225,143 +2272,143 @@
       <c r="K15" s="18">
         <v>905.7144</v>
       </c>
-      <c r="L15" s="19" t="s">
+      <c r="L15" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M15" s="19" t="s">
+      <c r="M15" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N15" s="20">
+      <c r="N15" s="18">
         <v>13.92</v>
       </c>
-      <c r="O15" s="21">
+      <c r="O15" s="19">
         <v>3</v>
       </c>
-      <c r="P15" s="20">
+      <c r="P15" s="18">
         <v>13.5</v>
       </c>
-      <c r="Q15" s="20">
+      <c r="Q15" s="18">
         <v>1215</v>
       </c>
-      <c r="R15" s="20">
+      <c r="R15" s="18">
         <v>1215</v>
       </c>
-      <c r="S15" s="20">
+      <c r="S15" s="18">
         <v>1147.5925</v>
       </c>
-      <c r="T15" s="16" t="s">
+      <c r="T15" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U15" s="16" t="s">
+      <c r="U15" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V15" s="20">
+      <c r="V15" s="18">
+        <v>13.35</v>
+      </c>
+      <c r="W15" s="19">
+        <v>8</v>
+      </c>
+      <c r="X15" s="18">
+        <v>12.282</v>
+      </c>
+      <c r="Y15" s="18">
+        <v>1105.38</v>
+      </c>
+      <c r="Z15" s="18">
+        <v>1105.38</v>
+      </c>
+      <c r="AA15" s="18">
+        <v>1023.6122</v>
+      </c>
+      <c r="AB15" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC15" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD15" s="18">
+        <v>15.34</v>
+      </c>
+      <c r="AE15" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF15" s="18">
+        <v>13.81</v>
+      </c>
+      <c r="AG15" s="18">
+        <v>1242.9</v>
+      </c>
+      <c r="AH15" s="18">
+        <v>1242.9</v>
+      </c>
+      <c r="AI15" s="18">
+        <v>1104.9892</v>
+      </c>
+      <c r="AJ15" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK15" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL15" s="18">
+        <v>12.92</v>
+      </c>
+      <c r="AM15" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN15" s="18">
+        <v>11.37</v>
+      </c>
+      <c r="AO15" s="18">
+        <v>1023.3</v>
+      </c>
+      <c r="AP15" s="18">
+        <v>1023.3</v>
+      </c>
+      <c r="AQ15" s="18">
+        <v>985.4519</v>
+      </c>
+      <c r="AR15" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS15" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT15" s="21">
         <v>14.77</v>
       </c>
-      <c r="W15" s="21">
+      <c r="AU15" s="22">
         <v>6</v>
       </c>
-      <c r="X15" s="20">
+      <c r="AV15" s="21">
         <v>13.88</v>
       </c>
-      <c r="Y15" s="20">
+      <c r="AW15" s="21">
         <v>1249.2</v>
       </c>
-      <c r="Z15" s="20">
+      <c r="AX15" s="21">
         <v>1249.2</v>
       </c>
-      <c r="AA15" s="20">
+      <c r="AY15" s="21">
         <v>1133.6918</v>
       </c>
-      <c r="AB15" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC15" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD15" s="20">
-        <v>13.35</v>
-      </c>
-      <c r="AE15" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF15" s="20">
-        <v>12.282</v>
-      </c>
-      <c r="AG15" s="20">
-        <v>1105.38</v>
-      </c>
-      <c r="AH15" s="20">
-        <v>1105.38</v>
-      </c>
-      <c r="AI15" s="20">
-        <v>1023.6122</v>
-      </c>
-      <c r="AJ15" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK15" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL15" s="20">
-        <v>15.34</v>
-      </c>
-      <c r="AM15" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN15" s="20">
-        <v>13.81</v>
-      </c>
-      <c r="AO15" s="20">
-        <v>1242.9</v>
-      </c>
-      <c r="AP15" s="20">
-        <v>1242.9</v>
-      </c>
-      <c r="AQ15" s="20">
-        <v>1104.9892</v>
-      </c>
-      <c r="AR15" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS15" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT15" s="20">
-        <v>12.92</v>
-      </c>
-      <c r="AU15" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV15" s="20">
-        <v>11.37</v>
-      </c>
-      <c r="AW15" s="20">
-        <v>1023.3</v>
-      </c>
-      <c r="AX15" s="20">
-        <v>1023.3</v>
-      </c>
-      <c r="AY15" s="20">
-        <v>985.4519</v>
-      </c>
-      <c r="AZ15" s="16" t="s">
+      <c r="AZ15" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA15" s="16" t="s">
+      <c r="BA15" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB15" s="19" t="s">
-        <v>25</v>
+      <c r="BB15" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC15" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD15" s="18">
-        <v>940.5</v>
+        <v>80</v>
+      </c>
+      <c r="BD15" s="21">
+        <v>1133.6918</v>
       </c>
       <c r="BE15" s="17" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:57">
@@ -2369,10 +2416,10 @@
         <v>7</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D16" s="16" t="s">
         <v>46</v>
@@ -2398,143 +2445,143 @@
       <c r="K16" s="18">
         <v>1097.8356</v>
       </c>
-      <c r="L16" s="19" t="s">
+      <c r="L16" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M16" s="19" t="s">
+      <c r="M16" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N16" s="20">
+      <c r="N16" s="18">
         <v>27.44</v>
       </c>
-      <c r="O16" s="21">
+      <c r="O16" s="19">
         <v>3</v>
       </c>
-      <c r="P16" s="20">
+      <c r="P16" s="18">
         <v>26.62</v>
       </c>
-      <c r="Q16" s="20">
+      <c r="Q16" s="18">
         <v>1597.2</v>
       </c>
-      <c r="R16" s="20">
+      <c r="R16" s="18">
         <v>1597.2</v>
       </c>
-      <c r="S16" s="20">
+      <c r="S16" s="18">
         <v>1508.5882</v>
       </c>
-      <c r="T16" s="16" t="s">
+      <c r="T16" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U16" s="16" t="s">
+      <c r="U16" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V16" s="20">
+      <c r="V16" s="18">
+        <v>26.32</v>
+      </c>
+      <c r="W16" s="19">
+        <v>8</v>
+      </c>
+      <c r="X16" s="18">
+        <v>24.2144</v>
+      </c>
+      <c r="Y16" s="18">
+        <v>1452.864</v>
+      </c>
+      <c r="Z16" s="18">
+        <v>1452.864</v>
+      </c>
+      <c r="AA16" s="18">
+        <v>1345.3919</v>
+      </c>
+      <c r="AB16" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC16" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD16" s="18">
+        <v>30.24</v>
+      </c>
+      <c r="AE16" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF16" s="18">
+        <v>27.22</v>
+      </c>
+      <c r="AG16" s="18">
+        <v>1633.2</v>
+      </c>
+      <c r="AH16" s="18">
+        <v>1633.2</v>
+      </c>
+      <c r="AI16" s="18">
+        <v>1451.9819</v>
+      </c>
+      <c r="AJ16" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK16" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL16" s="18">
+        <v>25.48</v>
+      </c>
+      <c r="AM16" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN16" s="18">
+        <v>22.42</v>
+      </c>
+      <c r="AO16" s="18">
+        <v>1345.2</v>
+      </c>
+      <c r="AP16" s="18">
+        <v>1345.2</v>
+      </c>
+      <c r="AQ16" s="18">
+        <v>1295.446</v>
+      </c>
+      <c r="AR16" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS16" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT16" s="21">
         <v>29.12</v>
       </c>
-      <c r="W16" s="21">
+      <c r="AU16" s="22">
         <v>6</v>
       </c>
-      <c r="X16" s="20">
+      <c r="AV16" s="21">
         <v>27.37</v>
       </c>
-      <c r="Y16" s="20">
+      <c r="AW16" s="21">
         <v>1642.2</v>
       </c>
-      <c r="Z16" s="20">
+      <c r="AX16" s="21">
         <v>1642.2</v>
       </c>
-      <c r="AA16" s="20">
+      <c r="AY16" s="21">
         <v>1490.3527</v>
       </c>
-      <c r="AB16" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC16" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD16" s="20">
-        <v>26.32</v>
-      </c>
-      <c r="AE16" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF16" s="20">
-        <v>24.2144</v>
-      </c>
-      <c r="AG16" s="20">
-        <v>1452.864</v>
-      </c>
-      <c r="AH16" s="20">
-        <v>1452.864</v>
-      </c>
-      <c r="AI16" s="20">
-        <v>1345.3919</v>
-      </c>
-      <c r="AJ16" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK16" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL16" s="20">
-        <v>30.24</v>
-      </c>
-      <c r="AM16" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN16" s="20">
-        <v>27.22</v>
-      </c>
-      <c r="AO16" s="20">
-        <v>1633.2</v>
-      </c>
-      <c r="AP16" s="20">
-        <v>1633.2</v>
-      </c>
-      <c r="AQ16" s="20">
-        <v>1451.9819</v>
-      </c>
-      <c r="AR16" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS16" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT16" s="20">
-        <v>25.48</v>
-      </c>
-      <c r="AU16" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV16" s="20">
-        <v>22.42</v>
-      </c>
-      <c r="AW16" s="20">
-        <v>1345.2</v>
-      </c>
-      <c r="AX16" s="20">
-        <v>1345.2</v>
-      </c>
-      <c r="AY16" s="20">
-        <v>1295.446</v>
-      </c>
-      <c r="AZ16" s="16" t="s">
+      <c r="AZ16" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA16" s="16" t="s">
+      <c r="BA16" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB16" s="19" t="s">
-        <v>25</v>
+      <c r="BB16" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC16" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD16" s="18">
-        <v>1140</v>
+        <v>84</v>
+      </c>
+      <c r="BD16" s="21">
+        <v>1490.3527</v>
       </c>
       <c r="BE16" s="17" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:57">
@@ -2542,10 +2589,10 @@
         <v>8</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>46</v>
@@ -2553,161 +2600,161 @@
       <c r="E17" s="16">
         <v>40</v>
       </c>
-      <c r="F17" s="20">
+      <c r="F17" s="18">
         <v>150</v>
       </c>
-      <c r="G17" s="21">
+      <c r="G17" s="19">
         <v>5</v>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="18">
         <v>142.5</v>
       </c>
-      <c r="I17" s="20">
+      <c r="I17" s="18">
         <v>5700</v>
       </c>
-      <c r="J17" s="20">
+      <c r="J17" s="18">
         <v>5700</v>
       </c>
-      <c r="K17" s="20">
+      <c r="K17" s="18">
         <v>5489.1781</v>
       </c>
-      <c r="L17" s="16" t="s">
+      <c r="L17" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M17" s="16" t="s">
+      <c r="M17" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N17" s="20">
+      <c r="N17" s="18">
         <v>164.13</v>
       </c>
-      <c r="O17" s="21">
+      <c r="O17" s="19">
         <v>3</v>
       </c>
-      <c r="P17" s="20">
+      <c r="P17" s="18">
         <v>159.21</v>
       </c>
-      <c r="Q17" s="20">
+      <c r="Q17" s="18">
         <v>6368.4</v>
       </c>
-      <c r="R17" s="20">
+      <c r="R17" s="18">
         <v>6368.4</v>
       </c>
-      <c r="S17" s="20">
+      <c r="S17" s="18">
         <v>6015.0847</v>
       </c>
-      <c r="T17" s="16" t="s">
+      <c r="T17" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U17" s="16" t="s">
+      <c r="U17" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V17" s="20">
+      <c r="V17" s="18">
+        <v>157.43</v>
+      </c>
+      <c r="W17" s="19">
+        <v>8</v>
+      </c>
+      <c r="X17" s="18">
+        <v>144.8356</v>
+      </c>
+      <c r="Y17" s="18">
+        <v>5793.424</v>
+      </c>
+      <c r="Z17" s="18">
+        <v>5793.424</v>
+      </c>
+      <c r="AA17" s="18">
+        <v>5364.8693</v>
+      </c>
+      <c r="AB17" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC17" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD17" s="18">
+        <v>180.87</v>
+      </c>
+      <c r="AE17" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF17" s="18">
+        <v>162.78</v>
+      </c>
+      <c r="AG17" s="18">
+        <v>6511.2</v>
+      </c>
+      <c r="AH17" s="18">
+        <v>6511.2</v>
+      </c>
+      <c r="AI17" s="18">
+        <v>5788.7244</v>
+      </c>
+      <c r="AJ17" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK17" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL17" s="18">
+        <v>152.4</v>
+      </c>
+      <c r="AM17" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN17" s="18">
+        <v>134.11</v>
+      </c>
+      <c r="AO17" s="18">
+        <v>5364.4</v>
+      </c>
+      <c r="AP17" s="18">
+        <v>5364.4</v>
+      </c>
+      <c r="AQ17" s="18">
+        <v>5165.9907</v>
+      </c>
+      <c r="AR17" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS17" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT17" s="21">
         <v>174.17</v>
       </c>
-      <c r="W17" s="21">
+      <c r="AU17" s="22">
         <v>6</v>
       </c>
-      <c r="X17" s="20">
+      <c r="AV17" s="21">
         <v>163.72</v>
       </c>
-      <c r="Y17" s="20">
+      <c r="AW17" s="21">
         <v>6548.8</v>
       </c>
-      <c r="Z17" s="20">
+      <c r="AX17" s="21">
         <v>6548.8</v>
       </c>
-      <c r="AA17" s="20">
+      <c r="AY17" s="21">
         <v>5943.2603</v>
       </c>
-      <c r="AB17" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC17" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD17" s="20">
-        <v>157.43</v>
-      </c>
-      <c r="AE17" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF17" s="20">
-        <v>144.8356</v>
-      </c>
-      <c r="AG17" s="20">
-        <v>5793.424</v>
-      </c>
-      <c r="AH17" s="20">
-        <v>5793.424</v>
-      </c>
-      <c r="AI17" s="20">
-        <v>5364.8693</v>
-      </c>
-      <c r="AJ17" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK17" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL17" s="20">
-        <v>180.87</v>
-      </c>
-      <c r="AM17" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN17" s="20">
-        <v>162.78</v>
-      </c>
-      <c r="AO17" s="20">
-        <v>6511.2</v>
-      </c>
-      <c r="AP17" s="20">
-        <v>6511.2</v>
-      </c>
-      <c r="AQ17" s="20">
-        <v>5788.7244</v>
-      </c>
-      <c r="AR17" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS17" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT17" s="18">
-        <v>152.4</v>
-      </c>
-      <c r="AU17" s="19">
-        <v>12</v>
-      </c>
-      <c r="AV17" s="18">
-        <v>134.11</v>
-      </c>
-      <c r="AW17" s="18">
-        <v>5364.4</v>
-      </c>
-      <c r="AX17" s="18">
-        <v>5364.4</v>
-      </c>
-      <c r="AY17" s="18">
-        <v>5165.9907</v>
-      </c>
-      <c r="AZ17" s="19" t="s">
+      <c r="AZ17" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA17" s="19" t="s">
+      <c r="BA17" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB17" s="19" t="s">
-        <v>81</v>
+      <c r="BB17" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC17" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD17" s="18">
-        <v>5364.4</v>
+        <v>88</v>
+      </c>
+      <c r="BD17" s="21">
+        <v>5943.2603</v>
       </c>
       <c r="BE17" s="17" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:57">
@@ -2715,10 +2762,10 @@
         <v>9</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>46</v>
@@ -2744,143 +2791,143 @@
       <c r="K18" s="18">
         <v>503.1747</v>
       </c>
-      <c r="L18" s="19" t="s">
+      <c r="L18" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M18" s="19" t="s">
+      <c r="M18" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N18" s="20">
+      <c r="N18" s="18">
         <v>7.97</v>
       </c>
-      <c r="O18" s="21">
+      <c r="O18" s="19">
         <v>3</v>
       </c>
-      <c r="P18" s="20">
+      <c r="P18" s="18">
         <v>7.73</v>
       </c>
-      <c r="Q18" s="20">
+      <c r="Q18" s="18">
         <v>850.3</v>
       </c>
-      <c r="R18" s="20">
+      <c r="R18" s="18">
         <v>850.3</v>
       </c>
-      <c r="S18" s="20">
+      <c r="S18" s="18">
         <v>803.1258</v>
       </c>
-      <c r="T18" s="16" t="s">
+      <c r="T18" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U18" s="16" t="s">
+      <c r="U18" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V18" s="20">
+      <c r="V18" s="18">
+        <v>7.65</v>
+      </c>
+      <c r="W18" s="19">
+        <v>8</v>
+      </c>
+      <c r="X18" s="18">
+        <v>7.038</v>
+      </c>
+      <c r="Y18" s="18">
+        <v>774.1799999999999</v>
+      </c>
+      <c r="Z18" s="18">
+        <v>774.1799999999999</v>
+      </c>
+      <c r="AA18" s="18">
+        <v>716.9118999999999</v>
+      </c>
+      <c r="AB18" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC18" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD18" s="18">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="AE18" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF18" s="18">
+        <v>7.91</v>
+      </c>
+      <c r="AG18" s="18">
+        <v>870.1</v>
+      </c>
+      <c r="AH18" s="18">
+        <v>870.1</v>
+      </c>
+      <c r="AI18" s="18">
+        <v>773.5547</v>
+      </c>
+      <c r="AJ18" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK18" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL18" s="18">
+        <v>7.4</v>
+      </c>
+      <c r="AM18" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN18" s="18">
+        <v>6.51</v>
+      </c>
+      <c r="AO18" s="18">
+        <v>716.1</v>
+      </c>
+      <c r="AP18" s="18">
+        <v>716.1</v>
+      </c>
+      <c r="AQ18" s="18">
+        <v>689.6141</v>
+      </c>
+      <c r="AR18" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS18" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT18" s="21">
         <v>8.460000000000001</v>
       </c>
-      <c r="W18" s="21">
+      <c r="AU18" s="22">
         <v>6</v>
       </c>
-      <c r="X18" s="20">
+      <c r="AV18" s="21">
         <v>7.95</v>
       </c>
-      <c r="Y18" s="20">
+      <c r="AW18" s="21">
         <v>874.5</v>
       </c>
-      <c r="Z18" s="20">
+      <c r="AX18" s="21">
         <v>874.5</v>
       </c>
-      <c r="AA18" s="20">
+      <c r="AY18" s="21">
         <v>793.6387</v>
       </c>
-      <c r="AB18" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC18" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD18" s="20">
-        <v>7.65</v>
-      </c>
-      <c r="AE18" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF18" s="20">
-        <v>7.038</v>
-      </c>
-      <c r="AG18" s="20">
-        <v>774.1799999999999</v>
-      </c>
-      <c r="AH18" s="20">
-        <v>774.1799999999999</v>
-      </c>
-      <c r="AI18" s="20">
-        <v>716.9118999999999</v>
-      </c>
-      <c r="AJ18" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK18" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL18" s="20">
-        <v>8.789999999999999</v>
-      </c>
-      <c r="AM18" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN18" s="20">
-        <v>7.91</v>
-      </c>
-      <c r="AO18" s="20">
-        <v>870.1</v>
-      </c>
-      <c r="AP18" s="20">
-        <v>870.1</v>
-      </c>
-      <c r="AQ18" s="20">
-        <v>773.5547</v>
-      </c>
-      <c r="AR18" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS18" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT18" s="20">
-        <v>7.4</v>
-      </c>
-      <c r="AU18" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV18" s="20">
-        <v>6.51</v>
-      </c>
-      <c r="AW18" s="20">
-        <v>716.1</v>
-      </c>
-      <c r="AX18" s="20">
-        <v>716.1</v>
-      </c>
-      <c r="AY18" s="20">
-        <v>689.6141</v>
-      </c>
-      <c r="AZ18" s="16" t="s">
+      <c r="AZ18" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA18" s="16" t="s">
+      <c r="BA18" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB18" s="19" t="s">
-        <v>25</v>
+      <c r="BB18" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC18" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD18" s="18">
-        <v>522.5</v>
+        <v>92</v>
+      </c>
+      <c r="BD18" s="21">
+        <v>793.6387</v>
       </c>
       <c r="BE18" s="17" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:57">
@@ -2888,10 +2935,10 @@
         <v>10</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>46</v>
@@ -2899,161 +2946,161 @@
       <c r="E19" s="16">
         <v>110</v>
       </c>
-      <c r="F19" s="20">
+      <c r="F19" s="18">
         <v>30</v>
       </c>
-      <c r="G19" s="21">
+      <c r="G19" s="19">
         <v>3</v>
       </c>
-      <c r="H19" s="20">
+      <c r="H19" s="18">
         <v>29.1</v>
       </c>
-      <c r="I19" s="20">
+      <c r="I19" s="18">
         <v>3201</v>
       </c>
-      <c r="J19" s="20">
+      <c r="J19" s="18">
         <v>3201</v>
       </c>
-      <c r="K19" s="20">
+      <c r="K19" s="18">
         <v>3082.6068</v>
       </c>
-      <c r="L19" s="16" t="s">
+      <c r="L19" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M19" s="16" t="s">
+      <c r="M19" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N19" s="20">
+      <c r="N19" s="18">
         <v>34.27</v>
       </c>
-      <c r="O19" s="21">
+      <c r="O19" s="19">
         <v>1</v>
       </c>
-      <c r="P19" s="20">
+      <c r="P19" s="18">
         <v>33.93</v>
       </c>
-      <c r="Q19" s="20">
+      <c r="Q19" s="18">
         <v>3732.3</v>
       </c>
-      <c r="R19" s="20">
+      <c r="R19" s="18">
         <v>3732.3</v>
       </c>
-      <c r="S19" s="20">
+      <c r="S19" s="18">
         <v>3525.234</v>
       </c>
-      <c r="T19" s="16" t="s">
+      <c r="T19" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U19" s="16" t="s">
+      <c r="U19" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V19" s="20">
+      <c r="V19" s="18">
+        <v>32.87</v>
+      </c>
+      <c r="W19" s="19">
+        <v>6</v>
+      </c>
+      <c r="X19" s="18">
+        <v>30.8978</v>
+      </c>
+      <c r="Y19" s="18">
+        <v>3398.758</v>
+      </c>
+      <c r="Z19" s="18">
+        <v>3398.758</v>
+      </c>
+      <c r="AA19" s="18">
+        <v>3147.343</v>
+      </c>
+      <c r="AB19" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC19" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD19" s="18">
+        <v>37.76</v>
+      </c>
+      <c r="AE19" s="19">
+        <v>8</v>
+      </c>
+      <c r="AF19" s="18">
+        <v>34.74</v>
+      </c>
+      <c r="AG19" s="18">
+        <v>3821.4</v>
+      </c>
+      <c r="AH19" s="18">
+        <v>3821.4</v>
+      </c>
+      <c r="AI19" s="18">
+        <v>3397.3816</v>
+      </c>
+      <c r="AJ19" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK19" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL19" s="18">
+        <v>31.32</v>
+      </c>
+      <c r="AM19" s="19">
+        <v>10</v>
+      </c>
+      <c r="AN19" s="18">
+        <v>28.64</v>
+      </c>
+      <c r="AO19" s="18">
+        <v>3150.4</v>
+      </c>
+      <c r="AP19" s="18">
+        <v>3150.4</v>
+      </c>
+      <c r="AQ19" s="18">
+        <v>3033.8784</v>
+      </c>
+      <c r="AR19" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS19" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT19" s="21">
         <v>36.37</v>
       </c>
-      <c r="W19" s="21">
+      <c r="AU19" s="22">
         <v>4</v>
       </c>
-      <c r="X19" s="20">
+      <c r="AV19" s="21">
         <v>34.92</v>
       </c>
-      <c r="Y19" s="20">
+      <c r="AW19" s="21">
         <v>3841.2</v>
       </c>
-      <c r="Z19" s="20">
+      <c r="AX19" s="21">
         <v>3841.2</v>
       </c>
-      <c r="AA19" s="20">
+      <c r="AY19" s="21">
         <v>3486.0205</v>
       </c>
-      <c r="AB19" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC19" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD19" s="20">
-        <v>32.87</v>
-      </c>
-      <c r="AE19" s="21">
-        <v>6</v>
-      </c>
-      <c r="AF19" s="20">
-        <v>30.8978</v>
-      </c>
-      <c r="AG19" s="20">
-        <v>3398.758</v>
-      </c>
-      <c r="AH19" s="20">
-        <v>3398.758</v>
-      </c>
-      <c r="AI19" s="20">
-        <v>3147.343</v>
-      </c>
-      <c r="AJ19" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK19" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL19" s="20">
-        <v>37.76</v>
-      </c>
-      <c r="AM19" s="21">
-        <v>8</v>
-      </c>
-      <c r="AN19" s="20">
-        <v>34.74</v>
-      </c>
-      <c r="AO19" s="20">
-        <v>3821.4</v>
-      </c>
-      <c r="AP19" s="20">
-        <v>3821.4</v>
-      </c>
-      <c r="AQ19" s="20">
-        <v>3397.3816</v>
-      </c>
-      <c r="AR19" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS19" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT19" s="18">
-        <v>31.32</v>
-      </c>
-      <c r="AU19" s="19">
-        <v>10</v>
-      </c>
-      <c r="AV19" s="18">
-        <v>28.64</v>
-      </c>
-      <c r="AW19" s="18">
-        <v>3150.4</v>
-      </c>
-      <c r="AX19" s="18">
-        <v>3150.4</v>
-      </c>
-      <c r="AY19" s="18">
-        <v>3033.8784</v>
-      </c>
-      <c r="AZ19" s="19" t="s">
+      <c r="AZ19" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA19" s="19" t="s">
+      <c r="BA19" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB19" s="19" t="s">
-        <v>81</v>
+      <c r="BB19" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC19" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD19" s="18">
-        <v>3150.4</v>
+        <v>96</v>
+      </c>
+      <c r="BD19" s="21">
+        <v>3486.0205</v>
       </c>
       <c r="BE19" s="17" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:57">
@@ -3061,10 +3108,10 @@
         <v>11</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="D20" s="16" t="s">
         <v>46</v>
@@ -3090,143 +3137,143 @@
       <c r="K20" s="18">
         <v>1494.5973</v>
       </c>
-      <c r="L20" s="19" t="s">
+      <c r="L20" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M20" s="19" t="s">
+      <c r="M20" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N20" s="20">
+      <c r="N20" s="18">
         <v>15.68</v>
       </c>
-      <c r="O20" s="21">
+      <c r="O20" s="19">
         <v>1</v>
       </c>
-      <c r="P20" s="20">
+      <c r="P20" s="18">
         <v>15.52</v>
       </c>
-      <c r="Q20" s="20">
+      <c r="Q20" s="18">
         <v>2483.2</v>
       </c>
-      <c r="R20" s="20">
+      <c r="R20" s="18">
         <v>2483.2</v>
       </c>
-      <c r="S20" s="20">
+      <c r="S20" s="18">
         <v>2345.4334</v>
       </c>
-      <c r="T20" s="16" t="s">
+      <c r="T20" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U20" s="16" t="s">
+      <c r="U20" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V20" s="20">
+      <c r="V20" s="18">
+        <v>15.04</v>
+      </c>
+      <c r="W20" s="19">
+        <v>6</v>
+      </c>
+      <c r="X20" s="18">
+        <v>14.1376</v>
+      </c>
+      <c r="Y20" s="18">
+        <v>2262.016</v>
+      </c>
+      <c r="Z20" s="18">
+        <v>2262.016</v>
+      </c>
+      <c r="AA20" s="18">
+        <v>2094.6888</v>
+      </c>
+      <c r="AB20" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC20" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD20" s="18">
+        <v>17.28</v>
+      </c>
+      <c r="AE20" s="19">
+        <v>8</v>
+      </c>
+      <c r="AF20" s="18">
+        <v>15.9</v>
+      </c>
+      <c r="AG20" s="18">
+        <v>2544</v>
+      </c>
+      <c r="AH20" s="18">
+        <v>2544</v>
+      </c>
+      <c r="AI20" s="18">
+        <v>2261.7205</v>
+      </c>
+      <c r="AJ20" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK20" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL20" s="18">
+        <v>14.56</v>
+      </c>
+      <c r="AM20" s="19">
+        <v>10</v>
+      </c>
+      <c r="AN20" s="18">
+        <v>13.1</v>
+      </c>
+      <c r="AO20" s="18">
+        <v>2096</v>
+      </c>
+      <c r="AP20" s="18">
+        <v>2096</v>
+      </c>
+      <c r="AQ20" s="18">
+        <v>2018.4767</v>
+      </c>
+      <c r="AR20" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS20" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT20" s="21">
         <v>16.64</v>
       </c>
-      <c r="W20" s="21">
+      <c r="AU20" s="22">
         <v>4</v>
       </c>
-      <c r="X20" s="20">
+      <c r="AV20" s="21">
         <v>15.97</v>
       </c>
-      <c r="Y20" s="20">
+      <c r="AW20" s="21">
         <v>2555.2</v>
       </c>
-      <c r="Z20" s="20">
+      <c r="AX20" s="21">
         <v>2555.2</v>
       </c>
-      <c r="AA20" s="20">
+      <c r="AY20" s="21">
         <v>2318.9315</v>
       </c>
-      <c r="AB20" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC20" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD20" s="20">
-        <v>15.04</v>
-      </c>
-      <c r="AE20" s="21">
-        <v>6</v>
-      </c>
-      <c r="AF20" s="20">
-        <v>14.1376</v>
-      </c>
-      <c r="AG20" s="20">
-        <v>2262.016</v>
-      </c>
-      <c r="AH20" s="20">
-        <v>2262.016</v>
-      </c>
-      <c r="AI20" s="20">
-        <v>2094.6888</v>
-      </c>
-      <c r="AJ20" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK20" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL20" s="20">
-        <v>17.28</v>
-      </c>
-      <c r="AM20" s="21">
-        <v>8</v>
-      </c>
-      <c r="AN20" s="20">
-        <v>15.9</v>
-      </c>
-      <c r="AO20" s="20">
-        <v>2544</v>
-      </c>
-      <c r="AP20" s="20">
-        <v>2544</v>
-      </c>
-      <c r="AQ20" s="20">
-        <v>2261.7205</v>
-      </c>
-      <c r="AR20" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS20" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT20" s="20">
-        <v>14.56</v>
-      </c>
-      <c r="AU20" s="21">
-        <v>10</v>
-      </c>
-      <c r="AV20" s="20">
-        <v>13.1</v>
-      </c>
-      <c r="AW20" s="20">
-        <v>2096</v>
-      </c>
-      <c r="AX20" s="20">
-        <v>2096</v>
-      </c>
-      <c r="AY20" s="20">
-        <v>2018.4767</v>
-      </c>
-      <c r="AZ20" s="16" t="s">
+      <c r="AZ20" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA20" s="16" t="s">
+      <c r="BA20" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB20" s="19" t="s">
-        <v>25</v>
+      <c r="BB20" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC20" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD20" s="18">
-        <v>1552</v>
+        <v>100</v>
+      </c>
+      <c r="BD20" s="21">
+        <v>2318.9315</v>
       </c>
       <c r="BE20" s="17" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:57">
@@ -3234,10 +3281,10 @@
         <v>12</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>46</v>
@@ -3263,143 +3310,143 @@
       <c r="K21" s="18">
         <v>46.7062</v>
       </c>
-      <c r="L21" s="19" t="s">
+      <c r="L21" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M21" s="19" t="s">
+      <c r="M21" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N21" s="20">
+      <c r="N21" s="18">
         <v>12.11</v>
       </c>
-      <c r="O21" s="21">
+      <c r="O21" s="19">
         <v>1</v>
       </c>
-      <c r="P21" s="20">
+      <c r="P21" s="18">
         <v>11.99</v>
       </c>
-      <c r="Q21" s="20">
+      <c r="Q21" s="18">
         <v>59.95</v>
       </c>
-      <c r="R21" s="20">
+      <c r="R21" s="18">
         <v>59.95</v>
       </c>
-      <c r="S21" s="20">
+      <c r="S21" s="18">
         <v>56.624</v>
       </c>
-      <c r="T21" s="16" t="s">
+      <c r="T21" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U21" s="16" t="s">
+      <c r="U21" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V21" s="20">
+      <c r="V21" s="18">
+        <v>11.62</v>
+      </c>
+      <c r="W21" s="19">
+        <v>6</v>
+      </c>
+      <c r="X21" s="18">
+        <v>10.9228</v>
+      </c>
+      <c r="Y21" s="18">
+        <v>54.614</v>
+      </c>
+      <c r="Z21" s="18">
+        <v>54.614</v>
+      </c>
+      <c r="AA21" s="18">
+        <v>50.5741</v>
+      </c>
+      <c r="AB21" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC21" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD21" s="18">
+        <v>13.35</v>
+      </c>
+      <c r="AE21" s="19">
+        <v>8</v>
+      </c>
+      <c r="AF21" s="18">
+        <v>12.28</v>
+      </c>
+      <c r="AG21" s="18">
+        <v>61.4</v>
+      </c>
+      <c r="AH21" s="18">
+        <v>61.4</v>
+      </c>
+      <c r="AI21" s="18">
+        <v>54.5871</v>
+      </c>
+      <c r="AJ21" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK21" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL21" s="18">
+        <v>11.25</v>
+      </c>
+      <c r="AM21" s="19">
+        <v>10</v>
+      </c>
+      <c r="AN21" s="18">
+        <v>10.12</v>
+      </c>
+      <c r="AO21" s="18">
+        <v>50.6</v>
+      </c>
+      <c r="AP21" s="18">
+        <v>50.6</v>
+      </c>
+      <c r="AQ21" s="18">
+        <v>48.7285</v>
+      </c>
+      <c r="AR21" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS21" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT21" s="21">
         <v>12.85</v>
       </c>
-      <c r="W21" s="21">
+      <c r="AU21" s="22">
         <v>4</v>
       </c>
-      <c r="X21" s="20">
+      <c r="AV21" s="21">
         <v>12.34</v>
       </c>
-      <c r="Y21" s="20">
+      <c r="AW21" s="21">
         <v>61.7</v>
       </c>
-      <c r="Z21" s="20">
+      <c r="AX21" s="21">
         <v>61.7</v>
       </c>
-      <c r="AA21" s="20">
+      <c r="AY21" s="21">
         <v>55.9949</v>
       </c>
-      <c r="AB21" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC21" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD21" s="20">
-        <v>11.62</v>
-      </c>
-      <c r="AE21" s="21">
-        <v>6</v>
-      </c>
-      <c r="AF21" s="20">
-        <v>10.9228</v>
-      </c>
-      <c r="AG21" s="20">
-        <v>54.614</v>
-      </c>
-      <c r="AH21" s="20">
-        <v>54.614</v>
-      </c>
-      <c r="AI21" s="20">
-        <v>50.5741</v>
-      </c>
-      <c r="AJ21" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK21" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL21" s="20">
-        <v>13.35</v>
-      </c>
-      <c r="AM21" s="21">
-        <v>8</v>
-      </c>
-      <c r="AN21" s="20">
-        <v>12.28</v>
-      </c>
-      <c r="AO21" s="20">
-        <v>61.4</v>
-      </c>
-      <c r="AP21" s="20">
-        <v>61.4</v>
-      </c>
-      <c r="AQ21" s="20">
-        <v>54.5871</v>
-      </c>
-      <c r="AR21" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS21" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT21" s="20">
-        <v>11.25</v>
-      </c>
-      <c r="AU21" s="21">
-        <v>10</v>
-      </c>
-      <c r="AV21" s="20">
-        <v>10.12</v>
-      </c>
-      <c r="AW21" s="20">
-        <v>50.6</v>
-      </c>
-      <c r="AX21" s="20">
-        <v>50.6</v>
-      </c>
-      <c r="AY21" s="20">
-        <v>48.7285</v>
-      </c>
-      <c r="AZ21" s="16" t="s">
+      <c r="AZ21" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA21" s="16" t="s">
+      <c r="BA21" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB21" s="19" t="s">
-        <v>25</v>
+      <c r="BB21" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC21" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD21" s="18">
-        <v>48.5</v>
+        <v>104</v>
+      </c>
+      <c r="BD21" s="21">
+        <v>55.9949</v>
       </c>
       <c r="BE21" s="17" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:57">
@@ -3407,10 +3454,10 @@
         <v>13</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>46</v>
@@ -3436,143 +3483,143 @@
       <c r="K22" s="18">
         <v>228.7158</v>
       </c>
-      <c r="L22" s="19" t="s">
+      <c r="L22" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M22" s="19" t="s">
+      <c r="M22" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="20">
+      <c r="N22" s="18">
         <v>9.029999999999999</v>
       </c>
-      <c r="O22" s="21">
+      <c r="O22" s="19">
         <v>3</v>
       </c>
-      <c r="P22" s="20">
+      <c r="P22" s="18">
         <v>8.76</v>
       </c>
-      <c r="Q22" s="20">
+      <c r="Q22" s="18">
         <v>438</v>
       </c>
-      <c r="R22" s="20">
+      <c r="R22" s="18">
         <v>438</v>
       </c>
-      <c r="S22" s="20">
+      <c r="S22" s="18">
         <v>413.7</v>
       </c>
-      <c r="T22" s="16" t="s">
+      <c r="T22" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U22" s="16" t="s">
+      <c r="U22" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V22" s="20">
+      <c r="V22" s="18">
+        <v>8.66</v>
+      </c>
+      <c r="W22" s="19">
+        <v>8</v>
+      </c>
+      <c r="X22" s="18">
+        <v>7.9672</v>
+      </c>
+      <c r="Y22" s="18">
+        <v>398.36</v>
+      </c>
+      <c r="Z22" s="18">
+        <v>398.36</v>
+      </c>
+      <c r="AA22" s="18">
+        <v>368.8923</v>
+      </c>
+      <c r="AB22" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC22" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD22" s="18">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="AE22" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF22" s="18">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="AG22" s="18">
+        <v>448</v>
+      </c>
+      <c r="AH22" s="18">
+        <v>448</v>
+      </c>
+      <c r="AI22" s="18">
+        <v>398.2904</v>
+      </c>
+      <c r="AJ22" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK22" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL22" s="18">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="AM22" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN22" s="18">
+        <v>7.38</v>
+      </c>
+      <c r="AO22" s="18">
+        <v>369</v>
+      </c>
+      <c r="AP22" s="18">
+        <v>369</v>
+      </c>
+      <c r="AQ22" s="18">
+        <v>355.3521</v>
+      </c>
+      <c r="AR22" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS22" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT22" s="21">
         <v>9.58</v>
       </c>
-      <c r="W22" s="21">
+      <c r="AU22" s="22">
         <v>6</v>
       </c>
-      <c r="X22" s="20">
+      <c r="AV22" s="21">
         <v>9.01</v>
       </c>
-      <c r="Y22" s="20">
+      <c r="AW22" s="21">
         <v>450.5</v>
       </c>
-      <c r="Z22" s="20">
+      <c r="AX22" s="21">
         <v>450.5</v>
       </c>
-      <c r="AA22" s="20">
+      <c r="AY22" s="21">
         <v>408.8442</v>
       </c>
-      <c r="AB22" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC22" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD22" s="20">
-        <v>8.66</v>
-      </c>
-      <c r="AE22" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF22" s="20">
-        <v>7.9672</v>
-      </c>
-      <c r="AG22" s="20">
-        <v>398.36</v>
-      </c>
-      <c r="AH22" s="20">
-        <v>398.36</v>
-      </c>
-      <c r="AI22" s="20">
-        <v>368.8923</v>
-      </c>
-      <c r="AJ22" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK22" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL22" s="20">
-        <v>9.949999999999999</v>
-      </c>
-      <c r="AM22" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN22" s="20">
-        <v>8.960000000000001</v>
-      </c>
-      <c r="AO22" s="20">
-        <v>448</v>
-      </c>
-      <c r="AP22" s="20">
-        <v>448</v>
-      </c>
-      <c r="AQ22" s="20">
-        <v>398.2904</v>
-      </c>
-      <c r="AR22" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS22" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT22" s="20">
-        <v>8.390000000000001</v>
-      </c>
-      <c r="AU22" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV22" s="20">
-        <v>7.38</v>
-      </c>
-      <c r="AW22" s="20">
-        <v>369</v>
-      </c>
-      <c r="AX22" s="20">
-        <v>369</v>
-      </c>
-      <c r="AY22" s="20">
-        <v>355.3521</v>
-      </c>
-      <c r="AZ22" s="16" t="s">
+      <c r="AZ22" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA22" s="16" t="s">
+      <c r="BA22" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB22" s="19" t="s">
-        <v>25</v>
+      <c r="BB22" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC22" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD22" s="18">
-        <v>237.5</v>
+        <v>108</v>
+      </c>
+      <c r="BD22" s="21">
+        <v>408.8442</v>
       </c>
       <c r="BE22" s="17" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:57">
@@ -3580,10 +3627,10 @@
         <v>14</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="D23" s="16" t="s">
         <v>46</v>
@@ -3609,166 +3656,166 @@
       <c r="K23" s="18">
         <v>960.6061999999999</v>
       </c>
-      <c r="L23" s="19" t="s">
+      <c r="L23" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M23" s="19" t="s">
+      <c r="M23" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="N23" s="20">
+      <c r="N23" s="18">
         <v>21.24</v>
       </c>
-      <c r="O23" s="21">
+      <c r="O23" s="19">
         <v>3</v>
       </c>
-      <c r="P23" s="20">
+      <c r="P23" s="18">
         <v>20.6</v>
       </c>
-      <c r="Q23" s="20">
+      <c r="Q23" s="18">
         <v>1442</v>
       </c>
-      <c r="R23" s="20">
+      <c r="R23" s="18">
         <v>1442</v>
       </c>
-      <c r="S23" s="20">
+      <c r="S23" s="18">
         <v>1361.9986</v>
       </c>
-      <c r="T23" s="16" t="s">
+      <c r="T23" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="U23" s="16" t="s">
+      <c r="U23" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="V23" s="20">
+      <c r="V23" s="18">
+        <v>20.37</v>
+      </c>
+      <c r="W23" s="19">
+        <v>8</v>
+      </c>
+      <c r="X23" s="18">
+        <v>18.7404</v>
+      </c>
+      <c r="Y23" s="18">
+        <v>1311.828</v>
+      </c>
+      <c r="Z23" s="18">
+        <v>1311.828</v>
+      </c>
+      <c r="AA23" s="18">
+        <v>1214.7887</v>
+      </c>
+      <c r="AB23" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC23" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD23" s="18">
+        <v>23.4</v>
+      </c>
+      <c r="AE23" s="19">
+        <v>10</v>
+      </c>
+      <c r="AF23" s="18">
+        <v>21.06</v>
+      </c>
+      <c r="AG23" s="18">
+        <v>1474.2</v>
+      </c>
+      <c r="AH23" s="18">
+        <v>1474.2</v>
+      </c>
+      <c r="AI23" s="18">
+        <v>1310.6244</v>
+      </c>
+      <c r="AJ23" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK23" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL23" s="18">
+        <v>19.72</v>
+      </c>
+      <c r="AM23" s="19">
+        <v>12</v>
+      </c>
+      <c r="AN23" s="18">
+        <v>17.35</v>
+      </c>
+      <c r="AO23" s="18">
+        <v>1214.5</v>
+      </c>
+      <c r="AP23" s="18">
+        <v>1214.5</v>
+      </c>
+      <c r="AQ23" s="18">
+        <v>1169.5801</v>
+      </c>
+      <c r="AR23" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS23" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT23" s="21">
         <v>22.54</v>
       </c>
-      <c r="W23" s="21">
+      <c r="AU23" s="22">
         <v>6</v>
       </c>
-      <c r="X23" s="20">
+      <c r="AV23" s="21">
         <v>21.19</v>
       </c>
-      <c r="Y23" s="20">
+      <c r="AW23" s="21">
         <v>1483.3</v>
       </c>
-      <c r="Z23" s="20">
+      <c r="AX23" s="21">
         <v>1483.3</v>
       </c>
-      <c r="AA23" s="20">
+      <c r="AY23" s="21">
         <v>1346.1455</v>
       </c>
-      <c r="AB23" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC23" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD23" s="20">
-        <v>20.37</v>
-      </c>
-      <c r="AE23" s="21">
-        <v>8</v>
-      </c>
-      <c r="AF23" s="20">
-        <v>18.7404</v>
-      </c>
-      <c r="AG23" s="20">
-        <v>1311.828</v>
-      </c>
-      <c r="AH23" s="20">
-        <v>1311.828</v>
-      </c>
-      <c r="AI23" s="20">
-        <v>1214.7887</v>
-      </c>
-      <c r="AJ23" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK23" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AL23" s="20">
-        <v>23.4</v>
-      </c>
-      <c r="AM23" s="21">
-        <v>10</v>
-      </c>
-      <c r="AN23" s="20">
-        <v>21.06</v>
-      </c>
-      <c r="AO23" s="20">
-        <v>1474.2</v>
-      </c>
-      <c r="AP23" s="20">
-        <v>1474.2</v>
-      </c>
-      <c r="AQ23" s="20">
-        <v>1310.6244</v>
-      </c>
-      <c r="AR23" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS23" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT23" s="20">
-        <v>19.72</v>
-      </c>
-      <c r="AU23" s="21">
-        <v>12</v>
-      </c>
-      <c r="AV23" s="20">
-        <v>17.35</v>
-      </c>
-      <c r="AW23" s="20">
-        <v>1214.5</v>
-      </c>
-      <c r="AX23" s="20">
-        <v>1214.5</v>
-      </c>
-      <c r="AY23" s="20">
-        <v>1169.5801</v>
-      </c>
-      <c r="AZ23" s="16" t="s">
+      <c r="AZ23" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="BA23" s="16" t="s">
+      <c r="BA23" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="BB23" s="19" t="s">
-        <v>25</v>
+      <c r="BB23" s="22" t="s">
+        <v>59</v>
       </c>
       <c r="BC23" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="BD23" s="18">
-        <v>997.5</v>
+        <v>112</v>
+      </c>
+      <c r="BD23" s="21">
+        <v>1346.1455</v>
       </c>
       <c r="BE23" s="17" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="1:57">
-      <c r="A25" s="19"/>
-      <c r="B25" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="D25" s="23"/>
-      <c r="E25" s="22" t="s">
-        <v>102</v>
+      <c r="A25" s="22"/>
+      <c r="B25" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="D25" s="20"/>
+      <c r="E25" s="23" t="s">
+        <v>115</v>
       </c>
       <c r="G25" s="24"/>
-      <c r="H25" s="22" t="s">
-        <v>103</v>
+      <c r="H25" s="23" t="s">
+        <v>116</v>
       </c>
       <c r="J25" s="25"/>
-      <c r="K25" s="22" t="s">
-        <v>104</v>
+      <c r="K25" s="23" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:57">
       <c r="A28" s="3" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -3776,7 +3823,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -3784,7 +3831,7 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
@@ -3792,7 +3839,7 @@
       <c r="Q28" s="3"/>
       <c r="R28" s="3"/>
       <c r="S28" s="3" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
@@ -3802,7 +3849,7 @@
     </row>
     <row r="29" spans="1:57">
       <c r="A29" s="5" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -3810,16 +3857,16 @@
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
       <c r="G29" s="26" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="H29" s="26" t="s">
         <v>22</v>
       </c>
       <c r="I29" s="26" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="N29" s="5"/>
       <c r="O29" s="5"/>
@@ -3827,7 +3874,7 @@
       <c r="Q29" s="5"/>
       <c r="R29" s="5"/>
       <c r="S29" s="5" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="T29" s="5"/>
       <c r="U29" s="5"/>
@@ -3843,13 +3890,13 @@
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
       <c r="G30" s="16" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="H30" s="17" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I30" s="17" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="M30" s="5"/>
       <c r="N30" s="5"/>
@@ -3872,13 +3919,13 @@
       <c r="E31" s="5"/>
       <c r="F31" s="5"/>
       <c r="G31" s="16" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="H31" s="17" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="I31" s="17" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
@@ -3954,11 +4001,11 @@
       <c r="X34" s="5"/>
     </row>
     <row r="36" spans="1:24">
-      <c r="A36" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="K36" s="22" t="s">
-        <v>116</v>
+      <c r="A36" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="K36" s="23" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rapor içeriğine ekleme yapılıyor.
</commit_message>
<xml_diff>
--- a/backend/app/temp/mukayese_raporu.xlsx
+++ b/backend/app/temp/mukayese_raporu.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="115">
   <si>
     <t>TEKLİF KARŞILAŞTIRMA RAPORU</t>
   </si>
@@ -46,7 +46,7 @@
     <t>En Avantajlı Firma Dağılımı</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik: 14</t>
+    <t>NOVA KURUMSAL TEDARİK: 14</t>
   </si>
   <si>
     <t>Para Birimi</t>
@@ -64,7 +64,7 @@
     <t>07.05.2026</t>
   </si>
   <si>
-    <t>20:28</t>
+    <t>21:09</t>
   </si>
   <si>
     <t>Bilgilendirme</t>
@@ -190,130 +190,127 @@
     <t>4 iş günü</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik</t>
-  </si>
-  <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 7,302.10 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 675.19 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 7,261.10 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 805.68 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>SİLGİ BÜYÜK</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 2,439.25 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%4 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 225.55 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 2,425.50 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%8 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 269.13 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>DEFTER A4</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 5,974.50 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 552.44 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 5,940.00 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 659.10 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>PERGEL</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 7,997.60 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 739.50 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 7,950.80 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 882.21 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>CETVEL</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 1,310.40 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 121.17 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 1,304.10 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 144.70 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>PİLOT KALEM</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 1,249.20 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 115.51 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 1,242.90 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 137.91 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>DOSYA KLASÖR</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 1,642.20 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 151.85 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 1,633.20 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 181.22 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>ZIMBA MAKİNESİ</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 6,548.80 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 605.54 TRY | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 6,511.20 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 722.48 TRY | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>silgi</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 874.50 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 80.86 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 870.10 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 96.55 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>defter</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 3,841.20 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%4 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 355.18 TRY | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 3,821.40 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%8 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 424.02 TRY | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>kalem tıraş</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 2,555.20 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%4 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 236.27 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 2,544.00 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%8 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 282.28 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>kalem</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 61.70 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%4 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 5.71 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 61.40 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%8 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 6.81 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>kurşun kalem</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 450.50 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 41.66 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 448.00 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 49.71 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>uçlu kalem</t>
   </si>
   <si>
-    <t>Teklif Zirve Tedarik önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 1,483.30 TRY | Vade: 75 gün | Termin: 4 gün</t>
-  </si>
-  <si>
-    <t>%6 iskonto | 75 gün vade | 4 gün termin | Vade avantajı: 137.15 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Kriter dışı: maksimum termin 7.0 gün, teklif 14 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün); Elendi: Maksimum termin şartını aşıyor (14 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | NOVA KURUMSAL TEDARİK elendi: Kriter dışı: maksimum termin 7.0 gün, teklif 10 gün; Elendi: Maksimum termin şartını aşıyor (10 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
+    <t>NOVA KURUMSAL TEDARİK önerildi. En düşük değerlendirilmiş maliyet ve satınalma kriter uygunluğu dikkate alındı. Net toplam: 1,474.20 TRY | Vade: 90 gün | Termin: 10 gün</t>
+  </si>
+  <si>
+    <t>%10 iskonto | 90 gün vade | 10 gün termin | Vade avantajı: 163.58 TRY | AYDIN KIRTASİYE LTD. ŞTİ. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | Teklif Kardelen Ofis elendi: Kriter dışı: minimum vade 70.0 gün, teklif 30 gün; Elendi: Minimum vade şartını sağlamıyor (30 gün) | MAVİ OFİS TEDARİK A.Ş. elendi: Kriter dışı: minimum vade 70.0 gün, teklif 60 gün; Elendi: Minimum vade şartını sağlamıyor (60 gün) | BETA KIRTASİYE PAZARLAMA elendi: Kriter dışı: minimum vade 70.0 gün, teklif 45 gün; Elendi: Minimum vade şartını sağlamıyor (45 gün)</t>
   </si>
   <si>
     <t>Önerilen / en avantajlı teklif</t>
@@ -375,7 +372,7 @@
     <t>Rapor Oluşturan: Sistem</t>
   </si>
   <si>
-    <t>Rapor No: RPR-20260507-2028</t>
+    <t>Rapor No: RPR-20260507-2109</t>
   </si>
 </sst>
 </file>
@@ -584,7 +581,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -648,6 +645,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1417,28 +1417,28 @@
       <c r="AC10" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD10" s="18">
+      <c r="AD10" s="21">
         <v>19.68</v>
       </c>
-      <c r="AE10" s="19">
+      <c r="AE10" s="22">
         <v>10</v>
       </c>
-      <c r="AF10" s="18">
+      <c r="AF10" s="21">
         <v>17.71</v>
       </c>
-      <c r="AG10" s="18">
+      <c r="AG10" s="21">
         <v>7261.1</v>
       </c>
-      <c r="AH10" s="18">
+      <c r="AH10" s="21">
         <v>7261.1</v>
       </c>
-      <c r="AI10" s="18">
+      <c r="AI10" s="21">
         <v>6455.4163</v>
       </c>
-      <c r="AJ10" s="20" t="s">
+      <c r="AJ10" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK10" s="20" t="s">
+      <c r="AK10" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL10" s="18">
@@ -1465,41 +1465,41 @@
       <c r="AS10" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT10" s="21">
+      <c r="AT10" s="23">
         <v>18.95</v>
       </c>
-      <c r="AU10" s="22">
+      <c r="AU10" s="19">
         <v>6</v>
       </c>
-      <c r="AV10" s="21">
+      <c r="AV10" s="23">
         <v>17.81</v>
       </c>
-      <c r="AW10" s="21">
+      <c r="AW10" s="23">
         <v>7302.1</v>
       </c>
-      <c r="AX10" s="21">
+      <c r="AX10" s="23">
         <v>7302.1</v>
       </c>
-      <c r="AY10" s="21">
+      <c r="AY10" s="23">
         <v>6626.9058</v>
       </c>
-      <c r="AZ10" s="22" t="s">
+      <c r="AZ10" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA10" s="22" t="s">
+      <c r="BA10" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB10" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="BC10" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="BC10" s="17" t="s">
+      <c r="BD10" s="21">
+        <v>6455.4163</v>
+      </c>
+      <c r="BE10" s="17" t="s">
         <v>59</v>
-      </c>
-      <c r="BD10" s="21">
-        <v>6626.9058</v>
-      </c>
-      <c r="BE10" s="17" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:57">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>45</v>
@@ -1588,28 +1588,28 @@
       <c r="AC11" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD11" s="18">
+      <c r="AD11" s="21">
         <v>9.59</v>
       </c>
-      <c r="AE11" s="19">
+      <c r="AE11" s="22">
         <v>8</v>
       </c>
-      <c r="AF11" s="18">
+      <c r="AF11" s="21">
         <v>8.82</v>
       </c>
-      <c r="AG11" s="18">
+      <c r="AG11" s="21">
         <v>2425.5</v>
       </c>
-      <c r="AH11" s="18">
+      <c r="AH11" s="21">
         <v>2425.5</v>
       </c>
-      <c r="AI11" s="18">
+      <c r="AI11" s="21">
         <v>2156.3692</v>
       </c>
-      <c r="AJ11" s="20" t="s">
+      <c r="AJ11" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK11" s="20" t="s">
+      <c r="AK11" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL11" s="18">
@@ -1636,41 +1636,41 @@
       <c r="AS11" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT11" s="21">
+      <c r="AT11" s="23">
         <v>9.24</v>
       </c>
-      <c r="AU11" s="22">
+      <c r="AU11" s="19">
         <v>4</v>
       </c>
-      <c r="AV11" s="21">
+      <c r="AV11" s="23">
         <v>8.869999999999999</v>
       </c>
-      <c r="AW11" s="21">
+      <c r="AW11" s="23">
         <v>2439.25</v>
       </c>
-      <c r="AX11" s="21">
+      <c r="AX11" s="23">
         <v>2439.25</v>
       </c>
-      <c r="AY11" s="21">
+      <c r="AY11" s="23">
         <v>2213.7029</v>
       </c>
-      <c r="AZ11" s="22" t="s">
+      <c r="AZ11" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA11" s="22" t="s">
+      <c r="BA11" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB11" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC11" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="BD11" s="21">
+        <v>2156.3692</v>
+      </c>
+      <c r="BE11" s="17" t="s">
         <v>62</v>
-      </c>
-      <c r="BD11" s="21">
-        <v>2213.7029</v>
-      </c>
-      <c r="BE11" s="17" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:57">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D12" s="16" t="s">
         <v>45</v>
@@ -1759,28 +1759,28 @@
       <c r="AC12" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD12" s="18">
+      <c r="AD12" s="21">
         <v>44</v>
       </c>
-      <c r="AE12" s="19">
+      <c r="AE12" s="22">
         <v>10</v>
       </c>
-      <c r="AF12" s="18">
+      <c r="AF12" s="21">
         <v>39.6</v>
       </c>
-      <c r="AG12" s="18">
+      <c r="AG12" s="21">
         <v>5940</v>
       </c>
-      <c r="AH12" s="18">
+      <c r="AH12" s="21">
         <v>5940</v>
       </c>
-      <c r="AI12" s="18">
+      <c r="AI12" s="21">
         <v>5280.9041</v>
       </c>
-      <c r="AJ12" s="20" t="s">
+      <c r="AJ12" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK12" s="20" t="s">
+      <c r="AK12" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL12" s="18">
@@ -1807,41 +1807,41 @@
       <c r="AS12" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT12" s="21">
+      <c r="AT12" s="23">
         <v>42.37</v>
       </c>
-      <c r="AU12" s="22">
+      <c r="AU12" s="19">
         <v>6</v>
       </c>
-      <c r="AV12" s="21">
+      <c r="AV12" s="23">
         <v>39.83</v>
       </c>
-      <c r="AW12" s="21">
+      <c r="AW12" s="23">
         <v>5974.5</v>
       </c>
-      <c r="AX12" s="21">
+      <c r="AX12" s="23">
         <v>5974.5</v>
       </c>
-      <c r="AY12" s="21">
+      <c r="AY12" s="23">
         <v>5422.0634</v>
       </c>
-      <c r="AZ12" s="22" t="s">
+      <c r="AZ12" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA12" s="22" t="s">
+      <c r="BA12" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB12" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC12" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="BD12" s="21">
+        <v>5280.9041</v>
+      </c>
+      <c r="BE12" s="17" t="s">
         <v>65</v>
-      </c>
-      <c r="BD12" s="21">
-        <v>5422.0634</v>
-      </c>
-      <c r="BE12" s="17" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:57">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="B13" s="17"/>
       <c r="C13" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>45</v>
@@ -1930,28 +1930,28 @@
       <c r="AC13" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD13" s="18">
+      <c r="AD13" s="21">
         <v>33.98</v>
       </c>
-      <c r="AE13" s="19">
+      <c r="AE13" s="22">
         <v>10</v>
       </c>
-      <c r="AF13" s="18">
+      <c r="AF13" s="21">
         <v>30.58</v>
       </c>
-      <c r="AG13" s="18">
+      <c r="AG13" s="21">
         <v>7950.8</v>
       </c>
-      <c r="AH13" s="18">
+      <c r="AH13" s="21">
         <v>7950.8</v>
       </c>
-      <c r="AI13" s="18">
+      <c r="AI13" s="21">
         <v>7068.5879</v>
       </c>
-      <c r="AJ13" s="20" t="s">
+      <c r="AJ13" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK13" s="20" t="s">
+      <c r="AK13" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL13" s="18">
@@ -1978,41 +1978,41 @@
       <c r="AS13" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT13" s="21">
+      <c r="AT13" s="23">
         <v>32.72</v>
       </c>
-      <c r="AU13" s="22">
+      <c r="AU13" s="19">
         <v>6</v>
       </c>
-      <c r="AV13" s="21">
+      <c r="AV13" s="23">
         <v>30.76</v>
       </c>
-      <c r="AW13" s="21">
+      <c r="AW13" s="23">
         <v>7997.6</v>
       </c>
-      <c r="AX13" s="21">
+      <c r="AX13" s="23">
         <v>7997.6</v>
       </c>
-      <c r="AY13" s="21">
+      <c r="AY13" s="23">
         <v>7258.0959</v>
       </c>
-      <c r="AZ13" s="22" t="s">
+      <c r="AZ13" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA13" s="22" t="s">
+      <c r="BA13" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB13" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC13" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="BD13" s="21">
+        <v>7068.5879</v>
+      </c>
+      <c r="BE13" s="17" t="s">
         <v>68</v>
-      </c>
-      <c r="BD13" s="21">
-        <v>7258.0959</v>
-      </c>
-      <c r="BE13" s="17" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:57">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>45</v>
@@ -2101,28 +2101,28 @@
       <c r="AC14" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD14" s="18">
+      <c r="AD14" s="21">
         <v>6.9</v>
       </c>
-      <c r="AE14" s="19">
+      <c r="AE14" s="22">
         <v>10</v>
       </c>
-      <c r="AF14" s="18">
+      <c r="AF14" s="21">
         <v>6.21</v>
       </c>
-      <c r="AG14" s="18">
+      <c r="AG14" s="21">
         <v>1304.1</v>
       </c>
-      <c r="AH14" s="18">
+      <c r="AH14" s="21">
         <v>1304.1</v>
       </c>
-      <c r="AI14" s="18">
+      <c r="AI14" s="21">
         <v>1159.3985</v>
       </c>
-      <c r="AJ14" s="20" t="s">
+      <c r="AJ14" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK14" s="20" t="s">
+      <c r="AK14" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL14" s="18">
@@ -2149,41 +2149,41 @@
       <c r="AS14" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT14" s="21">
+      <c r="AT14" s="23">
         <v>6.64</v>
       </c>
-      <c r="AU14" s="22">
+      <c r="AU14" s="19">
         <v>6</v>
       </c>
-      <c r="AV14" s="21">
+      <c r="AV14" s="23">
         <v>6.24</v>
       </c>
-      <c r="AW14" s="21">
+      <c r="AW14" s="23">
         <v>1310.4</v>
       </c>
-      <c r="AX14" s="21">
+      <c r="AX14" s="23">
         <v>1310.4</v>
       </c>
-      <c r="AY14" s="21">
+      <c r="AY14" s="23">
         <v>1189.2329</v>
       </c>
-      <c r="AZ14" s="22" t="s">
+      <c r="AZ14" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA14" s="22" t="s">
+      <c r="BA14" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB14" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC14" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="BD14" s="21">
+        <v>1159.3985</v>
+      </c>
+      <c r="BE14" s="17" t="s">
         <v>71</v>
-      </c>
-      <c r="BD14" s="21">
-        <v>1189.2329</v>
-      </c>
-      <c r="BE14" s="17" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:57">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>45</v>
@@ -2272,28 +2272,28 @@
       <c r="AC15" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD15" s="18">
+      <c r="AD15" s="21">
         <v>15.34</v>
       </c>
-      <c r="AE15" s="19">
+      <c r="AE15" s="22">
         <v>10</v>
       </c>
-      <c r="AF15" s="18">
+      <c r="AF15" s="21">
         <v>13.81</v>
       </c>
-      <c r="AG15" s="18">
+      <c r="AG15" s="21">
         <v>1242.9</v>
       </c>
-      <c r="AH15" s="18">
+      <c r="AH15" s="21">
         <v>1242.9</v>
       </c>
-      <c r="AI15" s="18">
+      <c r="AI15" s="21">
         <v>1104.9892</v>
       </c>
-      <c r="AJ15" s="20" t="s">
+      <c r="AJ15" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK15" s="20" t="s">
+      <c r="AK15" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL15" s="18">
@@ -2320,41 +2320,41 @@
       <c r="AS15" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT15" s="21">
+      <c r="AT15" s="23">
         <v>14.77</v>
       </c>
-      <c r="AU15" s="22">
+      <c r="AU15" s="19">
         <v>6</v>
       </c>
-      <c r="AV15" s="21">
+      <c r="AV15" s="23">
         <v>13.88</v>
       </c>
-      <c r="AW15" s="21">
+      <c r="AW15" s="23">
         <v>1249.2</v>
       </c>
-      <c r="AX15" s="21">
+      <c r="AX15" s="23">
         <v>1249.2</v>
       </c>
-      <c r="AY15" s="21">
+      <c r="AY15" s="23">
         <v>1133.6918</v>
       </c>
-      <c r="AZ15" s="22" t="s">
+      <c r="AZ15" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA15" s="22" t="s">
+      <c r="BA15" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB15" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC15" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="BD15" s="21">
+        <v>1104.9892</v>
+      </c>
+      <c r="BE15" s="17" t="s">
         <v>74</v>
-      </c>
-      <c r="BD15" s="21">
-        <v>1133.6918</v>
-      </c>
-      <c r="BE15" s="17" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:57">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D16" s="16" t="s">
         <v>45</v>
@@ -2443,28 +2443,28 @@
       <c r="AC16" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD16" s="18">
+      <c r="AD16" s="21">
         <v>30.24</v>
       </c>
-      <c r="AE16" s="19">
+      <c r="AE16" s="22">
         <v>10</v>
       </c>
-      <c r="AF16" s="18">
+      <c r="AF16" s="21">
         <v>27.22</v>
       </c>
-      <c r="AG16" s="18">
+      <c r="AG16" s="21">
         <v>1633.2</v>
       </c>
-      <c r="AH16" s="18">
+      <c r="AH16" s="21">
         <v>1633.2</v>
       </c>
-      <c r="AI16" s="18">
+      <c r="AI16" s="21">
         <v>1451.9819</v>
       </c>
-      <c r="AJ16" s="20" t="s">
+      <c r="AJ16" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK16" s="20" t="s">
+      <c r="AK16" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL16" s="18">
@@ -2491,41 +2491,41 @@
       <c r="AS16" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT16" s="21">
+      <c r="AT16" s="23">
         <v>29.12</v>
       </c>
-      <c r="AU16" s="22">
+      <c r="AU16" s="19">
         <v>6</v>
       </c>
-      <c r="AV16" s="21">
+      <c r="AV16" s="23">
         <v>27.37</v>
       </c>
-      <c r="AW16" s="21">
+      <c r="AW16" s="23">
         <v>1642.2</v>
       </c>
-      <c r="AX16" s="21">
+      <c r="AX16" s="23">
         <v>1642.2</v>
       </c>
-      <c r="AY16" s="21">
+      <c r="AY16" s="23">
         <v>1490.3527</v>
       </c>
-      <c r="AZ16" s="22" t="s">
+      <c r="AZ16" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA16" s="22" t="s">
+      <c r="BA16" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB16" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC16" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="BD16" s="21">
+        <v>1451.9819</v>
+      </c>
+      <c r="BE16" s="17" t="s">
         <v>77</v>
-      </c>
-      <c r="BD16" s="21">
-        <v>1490.3527</v>
-      </c>
-      <c r="BE16" s="17" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:57">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>45</v>
@@ -2614,28 +2614,28 @@
       <c r="AC17" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD17" s="18">
+      <c r="AD17" s="21">
         <v>180.87</v>
       </c>
-      <c r="AE17" s="19">
+      <c r="AE17" s="22">
         <v>10</v>
       </c>
-      <c r="AF17" s="18">
+      <c r="AF17" s="21">
         <v>162.78</v>
       </c>
-      <c r="AG17" s="18">
+      <c r="AG17" s="21">
         <v>6511.2</v>
       </c>
-      <c r="AH17" s="18">
+      <c r="AH17" s="21">
         <v>6511.2</v>
       </c>
-      <c r="AI17" s="18">
+      <c r="AI17" s="21">
         <v>5788.7244</v>
       </c>
-      <c r="AJ17" s="20" t="s">
+      <c r="AJ17" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK17" s="20" t="s">
+      <c r="AK17" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL17" s="18">
@@ -2662,41 +2662,41 @@
       <c r="AS17" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT17" s="21">
+      <c r="AT17" s="23">
         <v>174.17</v>
       </c>
-      <c r="AU17" s="22">
+      <c r="AU17" s="19">
         <v>6</v>
       </c>
-      <c r="AV17" s="21">
+      <c r="AV17" s="23">
         <v>163.72</v>
       </c>
-      <c r="AW17" s="21">
+      <c r="AW17" s="23">
         <v>6548.8</v>
       </c>
-      <c r="AX17" s="21">
+      <c r="AX17" s="23">
         <v>6548.8</v>
       </c>
-      <c r="AY17" s="21">
+      <c r="AY17" s="23">
         <v>5943.2603</v>
       </c>
-      <c r="AZ17" s="22" t="s">
+      <c r="AZ17" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA17" s="22" t="s">
+      <c r="BA17" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB17" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC17" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="BD17" s="21">
+        <v>5788.7244</v>
+      </c>
+      <c r="BE17" s="17" t="s">
         <v>80</v>
-      </c>
-      <c r="BD17" s="21">
-        <v>5943.2603</v>
-      </c>
-      <c r="BE17" s="17" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:57">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>45</v>
@@ -2785,28 +2785,28 @@
       <c r="AC18" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD18" s="18">
+      <c r="AD18" s="21">
         <v>8.789999999999999</v>
       </c>
-      <c r="AE18" s="19">
+      <c r="AE18" s="22">
         <v>10</v>
       </c>
-      <c r="AF18" s="18">
+      <c r="AF18" s="21">
         <v>7.91</v>
       </c>
-      <c r="AG18" s="18">
+      <c r="AG18" s="21">
         <v>870.1</v>
       </c>
-      <c r="AH18" s="18">
+      <c r="AH18" s="21">
         <v>870.1</v>
       </c>
-      <c r="AI18" s="18">
+      <c r="AI18" s="21">
         <v>773.5547</v>
       </c>
-      <c r="AJ18" s="20" t="s">
+      <c r="AJ18" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK18" s="20" t="s">
+      <c r="AK18" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL18" s="18">
@@ -2833,41 +2833,41 @@
       <c r="AS18" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT18" s="21">
+      <c r="AT18" s="23">
         <v>8.460000000000001</v>
       </c>
-      <c r="AU18" s="22">
+      <c r="AU18" s="19">
         <v>6</v>
       </c>
-      <c r="AV18" s="21">
+      <c r="AV18" s="23">
         <v>7.95</v>
       </c>
-      <c r="AW18" s="21">
+      <c r="AW18" s="23">
         <v>874.5</v>
       </c>
-      <c r="AX18" s="21">
+      <c r="AX18" s="23">
         <v>874.5</v>
       </c>
-      <c r="AY18" s="21">
+      <c r="AY18" s="23">
         <v>793.6387</v>
       </c>
-      <c r="AZ18" s="22" t="s">
+      <c r="AZ18" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA18" s="22" t="s">
+      <c r="BA18" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB18" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC18" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="BD18" s="21">
+        <v>773.5547</v>
+      </c>
+      <c r="BE18" s="17" t="s">
         <v>83</v>
-      </c>
-      <c r="BD18" s="21">
-        <v>793.6387</v>
-      </c>
-      <c r="BE18" s="17" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:57">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>45</v>
@@ -2956,28 +2956,28 @@
       <c r="AC19" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD19" s="18">
+      <c r="AD19" s="21">
         <v>37.76</v>
       </c>
-      <c r="AE19" s="19">
+      <c r="AE19" s="22">
         <v>8</v>
       </c>
-      <c r="AF19" s="18">
+      <c r="AF19" s="21">
         <v>34.74</v>
       </c>
-      <c r="AG19" s="18">
+      <c r="AG19" s="21">
         <v>3821.4</v>
       </c>
-      <c r="AH19" s="18">
+      <c r="AH19" s="21">
         <v>3821.4</v>
       </c>
-      <c r="AI19" s="18">
+      <c r="AI19" s="21">
         <v>3397.3816</v>
       </c>
-      <c r="AJ19" s="20" t="s">
+      <c r="AJ19" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK19" s="20" t="s">
+      <c r="AK19" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL19" s="18">
@@ -3004,41 +3004,41 @@
       <c r="AS19" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT19" s="21">
+      <c r="AT19" s="23">
         <v>36.37</v>
       </c>
-      <c r="AU19" s="22">
+      <c r="AU19" s="19">
         <v>4</v>
       </c>
-      <c r="AV19" s="21">
+      <c r="AV19" s="23">
         <v>34.92</v>
       </c>
-      <c r="AW19" s="21">
+      <c r="AW19" s="23">
         <v>3841.2</v>
       </c>
-      <c r="AX19" s="21">
+      <c r="AX19" s="23">
         <v>3841.2</v>
       </c>
-      <c r="AY19" s="21">
+      <c r="AY19" s="23">
         <v>3486.0205</v>
       </c>
-      <c r="AZ19" s="22" t="s">
+      <c r="AZ19" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA19" s="22" t="s">
+      <c r="BA19" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB19" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC19" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="BD19" s="21">
+        <v>3397.3816</v>
+      </c>
+      <c r="BE19" s="17" t="s">
         <v>86</v>
-      </c>
-      <c r="BD19" s="21">
-        <v>3486.0205</v>
-      </c>
-      <c r="BE19" s="17" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:57">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D20" s="16" t="s">
         <v>45</v>
@@ -3127,28 +3127,28 @@
       <c r="AC20" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD20" s="18">
+      <c r="AD20" s="21">
         <v>17.28</v>
       </c>
-      <c r="AE20" s="19">
+      <c r="AE20" s="22">
         <v>8</v>
       </c>
-      <c r="AF20" s="18">
+      <c r="AF20" s="21">
         <v>15.9</v>
       </c>
-      <c r="AG20" s="18">
+      <c r="AG20" s="21">
         <v>2544</v>
       </c>
-      <c r="AH20" s="18">
+      <c r="AH20" s="21">
         <v>2544</v>
       </c>
-      <c r="AI20" s="18">
+      <c r="AI20" s="21">
         <v>2261.7205</v>
       </c>
-      <c r="AJ20" s="20" t="s">
+      <c r="AJ20" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK20" s="20" t="s">
+      <c r="AK20" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL20" s="18">
@@ -3175,41 +3175,41 @@
       <c r="AS20" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT20" s="21">
+      <c r="AT20" s="23">
         <v>16.64</v>
       </c>
-      <c r="AU20" s="22">
+      <c r="AU20" s="19">
         <v>4</v>
       </c>
-      <c r="AV20" s="21">
+      <c r="AV20" s="23">
         <v>15.97</v>
       </c>
-      <c r="AW20" s="21">
+      <c r="AW20" s="23">
         <v>2555.2</v>
       </c>
-      <c r="AX20" s="21">
+      <c r="AX20" s="23">
         <v>2555.2</v>
       </c>
-      <c r="AY20" s="21">
+      <c r="AY20" s="23">
         <v>2318.9315</v>
       </c>
-      <c r="AZ20" s="22" t="s">
+      <c r="AZ20" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA20" s="22" t="s">
+      <c r="BA20" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB20" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC20" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="BD20" s="21">
+        <v>2261.7205</v>
+      </c>
+      <c r="BE20" s="17" t="s">
         <v>89</v>
-      </c>
-      <c r="BD20" s="21">
-        <v>2318.9315</v>
-      </c>
-      <c r="BE20" s="17" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:57">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>45</v>
@@ -3298,28 +3298,28 @@
       <c r="AC21" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD21" s="18">
+      <c r="AD21" s="21">
         <v>13.35</v>
       </c>
-      <c r="AE21" s="19">
+      <c r="AE21" s="22">
         <v>8</v>
       </c>
-      <c r="AF21" s="18">
+      <c r="AF21" s="21">
         <v>12.28</v>
       </c>
-      <c r="AG21" s="18">
+      <c r="AG21" s="21">
         <v>61.4</v>
       </c>
-      <c r="AH21" s="18">
+      <c r="AH21" s="21">
         <v>61.4</v>
       </c>
-      <c r="AI21" s="18">
+      <c r="AI21" s="21">
         <v>54.5871</v>
       </c>
-      <c r="AJ21" s="20" t="s">
+      <c r="AJ21" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK21" s="20" t="s">
+      <c r="AK21" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL21" s="18">
@@ -3346,41 +3346,41 @@
       <c r="AS21" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT21" s="21">
+      <c r="AT21" s="23">
         <v>12.85</v>
       </c>
-      <c r="AU21" s="22">
+      <c r="AU21" s="19">
         <v>4</v>
       </c>
-      <c r="AV21" s="21">
+      <c r="AV21" s="23">
         <v>12.34</v>
       </c>
-      <c r="AW21" s="21">
+      <c r="AW21" s="23">
         <v>61.7</v>
       </c>
-      <c r="AX21" s="21">
+      <c r="AX21" s="23">
         <v>61.7</v>
       </c>
-      <c r="AY21" s="21">
+      <c r="AY21" s="23">
         <v>55.9949</v>
       </c>
-      <c r="AZ21" s="22" t="s">
+      <c r="AZ21" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA21" s="22" t="s">
+      <c r="BA21" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB21" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC21" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="BD21" s="21">
+        <v>54.5871</v>
+      </c>
+      <c r="BE21" s="17" t="s">
         <v>92</v>
-      </c>
-      <c r="BD21" s="21">
-        <v>55.9949</v>
-      </c>
-      <c r="BE21" s="17" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:57">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>45</v>
@@ -3469,28 +3469,28 @@
       <c r="AC22" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD22" s="18">
+      <c r="AD22" s="21">
         <v>9.949999999999999</v>
       </c>
-      <c r="AE22" s="19">
+      <c r="AE22" s="22">
         <v>10</v>
       </c>
-      <c r="AF22" s="18">
+      <c r="AF22" s="21">
         <v>8.960000000000001</v>
       </c>
-      <c r="AG22" s="18">
+      <c r="AG22" s="21">
         <v>448</v>
       </c>
-      <c r="AH22" s="18">
+      <c r="AH22" s="21">
         <v>448</v>
       </c>
-      <c r="AI22" s="18">
+      <c r="AI22" s="21">
         <v>398.2904</v>
       </c>
-      <c r="AJ22" s="20" t="s">
+      <c r="AJ22" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK22" s="20" t="s">
+      <c r="AK22" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL22" s="18">
@@ -3517,41 +3517,41 @@
       <c r="AS22" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT22" s="21">
+      <c r="AT22" s="23">
         <v>9.58</v>
       </c>
-      <c r="AU22" s="22">
+      <c r="AU22" s="19">
         <v>6</v>
       </c>
-      <c r="AV22" s="21">
+      <c r="AV22" s="23">
         <v>9.01</v>
       </c>
-      <c r="AW22" s="21">
+      <c r="AW22" s="23">
         <v>450.5</v>
       </c>
-      <c r="AX22" s="21">
+      <c r="AX22" s="23">
         <v>450.5</v>
       </c>
-      <c r="AY22" s="21">
+      <c r="AY22" s="23">
         <v>408.8442</v>
       </c>
-      <c r="AZ22" s="22" t="s">
+      <c r="AZ22" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA22" s="22" t="s">
+      <c r="BA22" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB22" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC22" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="BD22" s="21">
+        <v>398.2904</v>
+      </c>
+      <c r="BE22" s="17" t="s">
         <v>95</v>
-      </c>
-      <c r="BD22" s="21">
-        <v>408.8442</v>
-      </c>
-      <c r="BE22" s="17" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:57">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="B23" s="17"/>
       <c r="C23" s="17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D23" s="16" t="s">
         <v>45</v>
@@ -3640,28 +3640,28 @@
       <c r="AC23" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AD23" s="18">
+      <c r="AD23" s="21">
         <v>23.4</v>
       </c>
-      <c r="AE23" s="19">
+      <c r="AE23" s="22">
         <v>10</v>
       </c>
-      <c r="AF23" s="18">
+      <c r="AF23" s="21">
         <v>21.06</v>
       </c>
-      <c r="AG23" s="18">
+      <c r="AG23" s="21">
         <v>1474.2</v>
       </c>
-      <c r="AH23" s="18">
+      <c r="AH23" s="21">
         <v>1474.2</v>
       </c>
-      <c r="AI23" s="18">
+      <c r="AI23" s="21">
         <v>1310.6244</v>
       </c>
-      <c r="AJ23" s="20" t="s">
+      <c r="AJ23" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="AK23" s="20" t="s">
+      <c r="AK23" s="22" t="s">
         <v>53</v>
       </c>
       <c r="AL23" s="18">
@@ -3688,64 +3688,64 @@
       <c r="AS23" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AT23" s="21">
+      <c r="AT23" s="23">
         <v>22.54</v>
       </c>
-      <c r="AU23" s="22">
+      <c r="AU23" s="19">
         <v>6</v>
       </c>
-      <c r="AV23" s="21">
+      <c r="AV23" s="23">
         <v>21.19</v>
       </c>
-      <c r="AW23" s="21">
+      <c r="AW23" s="23">
         <v>1483.3</v>
       </c>
-      <c r="AX23" s="21">
+      <c r="AX23" s="23">
         <v>1483.3</v>
       </c>
-      <c r="AY23" s="21">
+      <c r="AY23" s="23">
         <v>1346.1455</v>
       </c>
-      <c r="AZ23" s="22" t="s">
+      <c r="AZ23" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BA23" s="22" t="s">
+      <c r="BA23" s="16" t="s">
         <v>57</v>
       </c>
       <c r="BB23" s="22" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="BC23" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="BD23" s="21">
+        <v>1310.6244</v>
+      </c>
+      <c r="BE23" s="17" t="s">
         <v>98</v>
-      </c>
-      <c r="BD23" s="21">
-        <v>1346.1455</v>
-      </c>
-      <c r="BE23" s="17" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:57">
       <c r="A25" s="22"/>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="D25" s="20"/>
+      <c r="E25" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="D25" s="20"/>
-      <c r="E25" s="23" t="s">
+      <c r="G25" s="25"/>
+      <c r="H25" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="G25" s="24"/>
-      <c r="H25" s="23" t="s">
+      <c r="J25" s="26"/>
+      <c r="K25" s="24" t="s">
         <v>102</v>
-      </c>
-      <c r="J25" s="25"/>
-      <c r="K25" s="23" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:57">
       <c r="A28" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -3753,7 +3753,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -3761,7 +3761,7 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
@@ -3769,7 +3769,7 @@
       <c r="Q28" s="3"/>
       <c r="R28" s="3"/>
       <c r="S28" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
@@ -3779,24 +3779,24 @@
     </row>
     <row r="29" spans="1:57">
       <c r="A29" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
-      <c r="G29" s="26" t="s">
+      <c r="G29" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="H29" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="H29" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="26" t="s">
-        <v>108</v>
-      </c>
       <c r="M29" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N29" s="5"/>
       <c r="O29" s="5"/>
@@ -3804,7 +3804,7 @@
       <c r="Q29" s="5"/>
       <c r="R29" s="5"/>
       <c r="S29" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="T29" s="5"/>
       <c r="U29" s="5"/>
@@ -3820,7 +3820,7 @@
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
       <c r="G30" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
@@ -3924,11 +3924,11 @@
       <c r="X34" s="5"/>
     </row>
     <row r="36" spans="1:24">
-      <c r="A36" s="23" t="s">
+      <c r="A36" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="K36" s="24" t="s">
         <v>114</v>
-      </c>
-      <c r="K36" s="23" t="s">
-        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>